<commit_message>
feat(internal-quote): support UV painting prices and template import
</commit_message>
<xml_diff>
--- a/backend/app/data/internal_quote_import_templates/喷油报价单.xlsx
+++ b/backend/app/data/internal_quote_import_templates/喷油报价单.xlsx
@@ -1,10 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:dbsheet="http://web.wps.cn/et/2021/dbsheet" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
   <fileVersion appName="xl" lastEdited="3" lowestEdited="5" rupBuild="9302"/>
   <workbookPr/>
+  <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
+    <mc:Choice Requires="x15">
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Aalyaan\Desktop\内部报价各部门报价模板\"/>
+    </mc:Choice>
+  </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="23040" windowHeight="10500"/>
+    <workbookView windowWidth="24750" windowHeight="12060"/>
   </bookViews>
   <sheets>
     <sheet name="喷油0923" sheetId="1" r:id="rId1"/>
@@ -711,7 +716,7 @@
     <definedName name="Wire26_8in">#REF!</definedName>
     <definedName name="WORDREPORT">'[4]Home Page'!$AB$1</definedName>
     <definedName name="電子元件表1">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">喷油0923!$A$1:$U$41</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">喷油0923!$A$1:$W$41</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -731,7 +736,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="51" uniqueCount="46">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="48">
   <si>
     <t>第二代恐龙公园报价</t>
   </si>
@@ -755,6 +760,12 @@
   </si>
   <si>
     <t>移印单价</t>
+  </si>
+  <si>
+    <t>UV</t>
+  </si>
+  <si>
+    <t>UV单价</t>
   </si>
   <si>
     <t>散枪</t>
@@ -909,13 +920,13 @@
       <charset val="134"/>
     </font>
     <font>
-      <sz val="14"/>
+      <sz val="11"/>
       <color rgb="FFFF0000"/>
       <name val="宋体"/>
       <charset val="134"/>
     </font>
     <font>
-      <sz val="11"/>
+      <sz val="14"/>
       <color rgb="FFFF0000"/>
       <name val="宋体"/>
       <charset val="134"/>
@@ -1586,7 +1597,7 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="36">
+  <cellXfs count="33">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1620,6 +1631,9 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1632,6 +1646,9 @@
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
@@ -1644,6 +1661,12 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1653,46 +1676,25 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="2" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="4" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center" wrapText="1"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="1" fillId="3" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="0" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="5" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
   </cellXfs>
@@ -2749,24 +2751,24 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:W43"/>
-  <sheetFormatPr defaultColWidth="11.4537037037037" defaultRowHeight="40" customHeight="1"/>
+  <dimension ref="A1:Y43"/>
+  <sheetFormatPr defaultColWidth="11.45" defaultRowHeight="40" customHeight="1"/>
   <cols>
-    <col min="1" max="2" width="20.4444444444444" style="5" customWidth="1"/>
-    <col min="3" max="3" width="11.787037037037" style="5" customWidth="1"/>
-    <col min="4" max="5" width="6.62962962962963" style="5" customWidth="1"/>
+    <col min="1" max="2" width="20.4416666666667" style="5" customWidth="1"/>
+    <col min="3" max="3" width="11.7833333333333" style="5" customWidth="1"/>
+    <col min="4" max="5" width="6.63333333333333" style="5" customWidth="1"/>
     <col min="6" max="6" width="7.5" style="5" customWidth="1"/>
-    <col min="7" max="18" width="6.62962962962963" style="5" customWidth="1"/>
-    <col min="19" max="19" width="8.88888888888889" style="5" customWidth="1"/>
-    <col min="20" max="20" width="6.62962962962963" style="5" customWidth="1"/>
-    <col min="21" max="21" width="18.212962962963" style="5" customWidth="1"/>
-    <col min="22" max="22" width="11.4537037037037" style="1" customWidth="1"/>
-    <col min="23" max="23" width="11.4537037037037" style="6" customWidth="1"/>
-    <col min="24" max="16380" width="11.4537037037037" style="1" customWidth="1"/>
-    <col min="16381" max="16384" width="11.4537037037037" style="1"/>
+    <col min="7" max="20" width="6.63333333333333" style="5" customWidth="1"/>
+    <col min="21" max="21" width="8.89166666666667" style="5" customWidth="1"/>
+    <col min="22" max="22" width="6.63333333333333" style="5" customWidth="1"/>
+    <col min="23" max="23" width="18.2166666666667" style="5" customWidth="1"/>
+    <col min="24" max="24" width="11.45" style="1" customWidth="1"/>
+    <col min="25" max="25" width="11.45" style="6" customWidth="1"/>
+    <col min="26" max="16382" width="11.45" style="1" customWidth="1"/>
+    <col min="16383" max="16384" width="11.45" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" customHeight="1" spans="1:23">
+    <row r="1" s="1" customFormat="1" customHeight="1" spans="1:25">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -2790,9 +2792,11 @@
       <c r="S1" s="7"/>
       <c r="T1" s="7"/>
       <c r="U1" s="7"/>
-      <c r="W1" s="6"/>
+      <c r="V1" s="7"/>
+      <c r="W1" s="7"/>
+      <c r="Y1" s="6"/>
     </row>
-    <row r="2" s="2" customFormat="1" customHeight="1" spans="1:23">
+    <row r="2" s="2" customFormat="1" customHeight="1" spans="1:25">
       <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
@@ -2850,1331 +2854,1427 @@
       <c r="S2" s="10" t="s">
         <v>19</v>
       </c>
-      <c r="T2" s="8" t="s">
+      <c r="T2" s="9" t="s">
         <v>20</v>
       </c>
-      <c r="U2" s="8" t="s">
+      <c r="U2" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="W2" s="28"/>
+      <c r="V2" s="8" t="s">
+        <v>22</v>
+      </c>
+      <c r="W2" s="8" t="s">
+        <v>23</v>
+      </c>
+      <c r="Y2" s="11"/>
     </row>
-    <row r="3" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A3" s="11"/>
-      <c r="B3" s="11"/>
-      <c r="C3" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D3" s="13"/>
-      <c r="E3" s="14"/>
-      <c r="F3" s="14">
+    <row r="3" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A3" s="12"/>
+      <c r="B3" s="12"/>
+      <c r="C3" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D3" s="14"/>
+      <c r="E3" s="15"/>
+      <c r="F3" s="15">
         <v>2</v>
       </c>
-      <c r="G3" s="14">
+      <c r="G3" s="15">
         <v>0.15</v>
       </c>
-      <c r="H3" s="14"/>
-      <c r="I3" s="14"/>
-      <c r="J3" s="14"/>
-      <c r="K3" s="14"/>
-      <c r="L3" s="14"/>
-      <c r="M3" s="14"/>
-      <c r="N3" s="14"/>
-      <c r="O3" s="14"/>
-      <c r="P3" s="14"/>
-      <c r="Q3" s="14"/>
-      <c r="R3" s="14"/>
-      <c r="S3" s="14"/>
-      <c r="T3" s="14">
-        <f t="shared" ref="T3:T10" si="0">D3*E3+F3*G3+H3*I3+J3*K3+L3*M3+N3*O3+P3*Q3+R3*S3</f>
+      <c r="H3" s="15"/>
+      <c r="I3" s="15"/>
+      <c r="J3" s="15"/>
+      <c r="K3" s="15"/>
+      <c r="L3" s="15"/>
+      <c r="M3" s="15"/>
+      <c r="N3" s="15"/>
+      <c r="O3" s="15"/>
+      <c r="P3" s="15"/>
+      <c r="Q3" s="15"/>
+      <c r="R3" s="15"/>
+      <c r="S3" s="15"/>
+      <c r="T3" s="15"/>
+      <c r="U3" s="15"/>
+      <c r="V3" s="15">
+        <f>D3*E3+F3*G3+H3*I3+J3*K3+L3*M3+N3*O3+P3*Q3+R3*S3+T3*U3</f>
         <v>0.3</v>
       </c>
-      <c r="U3" s="14"/>
-      <c r="V3" s="1">
+      <c r="W3" s="15"/>
+      <c r="X3" s="1">
         <v>1.77</v>
       </c>
-      <c r="W3" s="29"/>
+      <c r="Y3" s="16"/>
     </row>
-    <row r="4" s="3" customFormat="1" ht="15" customHeight="1" spans="1:23">
-      <c r="A4" s="15"/>
-      <c r="B4" s="15"/>
-      <c r="C4" s="16"/>
-      <c r="D4" s="17"/>
-      <c r="E4" s="18"/>
-      <c r="F4" s="18"/>
-      <c r="G4" s="18"/>
-      <c r="H4" s="18"/>
-      <c r="I4" s="18"/>
-      <c r="J4" s="18"/>
-      <c r="K4" s="18"/>
-      <c r="L4" s="18"/>
-      <c r="M4" s="18"/>
-      <c r="N4" s="18"/>
-      <c r="O4" s="18"/>
-      <c r="P4" s="18"/>
-      <c r="Q4" s="18"/>
-      <c r="R4" s="18"/>
-      <c r="S4" s="18"/>
-      <c r="T4" s="18"/>
-      <c r="U4" s="18"/>
-      <c r="W4" s="30"/>
+    <row r="4" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
+      <c r="A4" s="17"/>
+      <c r="B4" s="17"/>
+      <c r="C4" s="18"/>
+      <c r="D4" s="19"/>
+      <c r="E4" s="20"/>
+      <c r="F4" s="20"/>
+      <c r="G4" s="20"/>
+      <c r="H4" s="20"/>
+      <c r="I4" s="20"/>
+      <c r="J4" s="20"/>
+      <c r="K4" s="20"/>
+      <c r="L4" s="20"/>
+      <c r="M4" s="20"/>
+      <c r="N4" s="20"/>
+      <c r="O4" s="20"/>
+      <c r="P4" s="20"/>
+      <c r="Q4" s="20"/>
+      <c r="R4" s="20"/>
+      <c r="S4" s="20"/>
+      <c r="T4" s="20"/>
+      <c r="U4" s="20"/>
+      <c r="V4" s="20"/>
+      <c r="W4" s="20"/>
+      <c r="Y4" s="21"/>
     </row>
-    <row r="5" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A5" s="14"/>
-      <c r="B5" s="14"/>
-      <c r="C5" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D5" s="14"/>
-      <c r="E5" s="14"/>
-      <c r="F5" s="14">
+    <row r="5" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A5" s="15"/>
+      <c r="B5" s="15"/>
+      <c r="C5" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D5" s="15"/>
+      <c r="E5" s="15"/>
+      <c r="F5" s="15">
         <v>2</v>
       </c>
-      <c r="G5" s="14">
+      <c r="G5" s="15">
         <v>0.05</v>
       </c>
-      <c r="H5" s="14"/>
-      <c r="I5" s="14"/>
-      <c r="J5" s="14"/>
-      <c r="K5" s="14"/>
-      <c r="L5" s="14"/>
-      <c r="M5" s="14"/>
-      <c r="N5" s="14"/>
-      <c r="O5" s="14"/>
-      <c r="P5" s="14"/>
-      <c r="Q5" s="14"/>
-      <c r="R5" s="14"/>
-      <c r="S5" s="14"/>
-      <c r="T5" s="14">
+      <c r="H5" s="15"/>
+      <c r="I5" s="15"/>
+      <c r="J5" s="15"/>
+      <c r="K5" s="15"/>
+      <c r="L5" s="15"/>
+      <c r="M5" s="15"/>
+      <c r="N5" s="15"/>
+      <c r="O5" s="15"/>
+      <c r="P5" s="15"/>
+      <c r="Q5" s="15"/>
+      <c r="R5" s="15"/>
+      <c r="S5" s="15"/>
+      <c r="T5" s="15"/>
+      <c r="U5" s="15"/>
+      <c r="V5" s="15">
+        <f>D5*E5+F5*G5+H5*I5+J5*K5+L5*M5+N5*O5+P5*Q5+R5*S5+T5*U5</f>
+        <v>0.1</v>
+      </c>
+      <c r="W5" s="15"/>
+      <c r="Y5" s="16"/>
+    </row>
+    <row r="6" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A6" s="15"/>
+      <c r="B6" s="15"/>
+      <c r="C6" s="15" t="s">
+        <v>26</v>
+      </c>
+      <c r="D6" s="15"/>
+      <c r="E6" s="15"/>
+      <c r="F6" s="15">
+        <v>4</v>
+      </c>
+      <c r="G6" s="15">
+        <v>0.05</v>
+      </c>
+      <c r="H6" s="15"/>
+      <c r="I6" s="15"/>
+      <c r="J6" s="15"/>
+      <c r="K6" s="15"/>
+      <c r="L6" s="15"/>
+      <c r="M6" s="15"/>
+      <c r="N6" s="15"/>
+      <c r="O6" s="15"/>
+      <c r="P6" s="15"/>
+      <c r="Q6" s="15"/>
+      <c r="R6" s="15"/>
+      <c r="S6" s="15"/>
+      <c r="T6" s="15"/>
+      <c r="U6" s="15"/>
+      <c r="V6" s="15">
+        <f>D6*E6+F6*G6+H6*I6+J6*K6+L6*M6+N6*O6+P6*Q6+R6*S6+T6*U6</f>
+        <v>0.2</v>
+      </c>
+      <c r="W6" s="15"/>
+      <c r="Y6" s="16"/>
+    </row>
+    <row r="7" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A7" s="15"/>
+      <c r="B7" s="15"/>
+      <c r="C7" s="15" t="s">
+        <v>27</v>
+      </c>
+      <c r="D7" s="15"/>
+      <c r="E7" s="15"/>
+      <c r="F7" s="15">
+        <v>2</v>
+      </c>
+      <c r="G7" s="15">
+        <v>0.05</v>
+      </c>
+      <c r="H7" s="15"/>
+      <c r="I7" s="15"/>
+      <c r="J7" s="15"/>
+      <c r="K7" s="15"/>
+      <c r="L7" s="15"/>
+      <c r="M7" s="15"/>
+      <c r="N7" s="15"/>
+      <c r="O7" s="15"/>
+      <c r="P7" s="15"/>
+      <c r="Q7" s="15"/>
+      <c r="R7" s="15"/>
+      <c r="S7" s="15"/>
+      <c r="T7" s="15"/>
+      <c r="U7" s="15"/>
+      <c r="V7" s="15">
+        <f t="shared" ref="V7:V12" si="0">D7*E7+F7*G7+H7*I7+J7*K7+L7*M7+N7*O7+P7*Q7+R7*S7+T7*U7</f>
+        <v>0.1</v>
+      </c>
+      <c r="W7" s="15"/>
+      <c r="Y7" s="16"/>
+    </row>
+    <row r="8" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A8" s="15"/>
+      <c r="B8" s="15"/>
+      <c r="C8" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="D8" s="15"/>
+      <c r="E8" s="15"/>
+      <c r="F8" s="15">
+        <v>2</v>
+      </c>
+      <c r="G8" s="15">
+        <v>0.05</v>
+      </c>
+      <c r="H8" s="15"/>
+      <c r="I8" s="15"/>
+      <c r="J8" s="15"/>
+      <c r="K8" s="15"/>
+      <c r="L8" s="15"/>
+      <c r="M8" s="15"/>
+      <c r="N8" s="15"/>
+      <c r="O8" s="15"/>
+      <c r="P8" s="15"/>
+      <c r="Q8" s="15"/>
+      <c r="R8" s="15"/>
+      <c r="S8" s="15"/>
+      <c r="T8" s="15"/>
+      <c r="U8" s="15"/>
+      <c r="V8" s="15">
         <f t="shared" si="0"/>
         <v>0.1</v>
       </c>
-      <c r="U5" s="14"/>
-      <c r="W5" s="29"/>
+      <c r="W8" s="15"/>
+      <c r="Y8" s="6"/>
     </row>
-    <row r="6" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A6" s="14"/>
-      <c r="B6" s="14"/>
-      <c r="C6" s="14" t="s">
-        <v>24</v>
-      </c>
-      <c r="D6" s="14"/>
-      <c r="E6" s="14"/>
-      <c r="F6" s="14">
-        <v>4</v>
-      </c>
-      <c r="G6" s="14">
+    <row r="9" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A9" s="15"/>
+      <c r="B9" s="15"/>
+      <c r="C9" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D9" s="15"/>
+      <c r="E9" s="15"/>
+      <c r="F9" s="15">
+        <v>1</v>
+      </c>
+      <c r="G9" s="15">
         <v>0.05</v>
       </c>
-      <c r="H6" s="14"/>
-      <c r="I6" s="14"/>
-      <c r="J6" s="14"/>
-      <c r="K6" s="14"/>
-      <c r="L6" s="14"/>
-      <c r="M6" s="14"/>
-      <c r="N6" s="14"/>
-      <c r="O6" s="14"/>
-      <c r="P6" s="14"/>
-      <c r="Q6" s="14"/>
-      <c r="R6" s="14"/>
-      <c r="S6" s="14"/>
-      <c r="T6" s="14">
+      <c r="H9" s="15"/>
+      <c r="I9" s="15"/>
+      <c r="J9" s="15"/>
+      <c r="K9" s="15"/>
+      <c r="L9" s="15"/>
+      <c r="M9" s="15"/>
+      <c r="N9" s="15"/>
+      <c r="O9" s="15"/>
+      <c r="P9" s="15"/>
+      <c r="Q9" s="15"/>
+      <c r="R9" s="15"/>
+      <c r="S9" s="15"/>
+      <c r="T9" s="15"/>
+      <c r="U9" s="15"/>
+      <c r="V9" s="15">
         <f t="shared" si="0"/>
-        <v>0.2</v>
-      </c>
-      <c r="U6" s="14"/>
-      <c r="W6" s="29"/>
+        <v>0.05</v>
+      </c>
+      <c r="W9" s="15"/>
+      <c r="Y9" s="6"/>
     </row>
-    <row r="7" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A7" s="14"/>
-      <c r="B7" s="14"/>
-      <c r="C7" s="14" t="s">
-        <v>25</v>
-      </c>
-      <c r="D7" s="14"/>
-      <c r="E7" s="14"/>
-      <c r="F7" s="14">
+    <row r="10" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A10" s="15"/>
+      <c r="B10" s="15"/>
+      <c r="C10" s="15" t="s">
+        <v>30</v>
+      </c>
+      <c r="D10" s="15"/>
+      <c r="E10" s="15"/>
+      <c r="F10" s="15"/>
+      <c r="G10" s="15"/>
+      <c r="H10" s="15"/>
+      <c r="I10" s="15"/>
+      <c r="J10" s="15">
         <v>2</v>
       </c>
-      <c r="G7" s="14">
-        <v>0.05</v>
-      </c>
-      <c r="H7" s="14"/>
-      <c r="I7" s="14"/>
-      <c r="J7" s="14"/>
-      <c r="K7" s="14"/>
-      <c r="L7" s="14"/>
-      <c r="M7" s="14"/>
-      <c r="N7" s="14"/>
-      <c r="O7" s="14"/>
-      <c r="P7" s="14"/>
-      <c r="Q7" s="14"/>
-      <c r="R7" s="14"/>
-      <c r="S7" s="14"/>
-      <c r="T7" s="14">
+      <c r="K10" s="15">
+        <v>0.08</v>
+      </c>
+      <c r="L10" s="15">
+        <v>1</v>
+      </c>
+      <c r="M10" s="15">
+        <v>0.08</v>
+      </c>
+      <c r="N10" s="15"/>
+      <c r="O10" s="15"/>
+      <c r="P10" s="15"/>
+      <c r="Q10" s="15"/>
+      <c r="R10" s="15"/>
+      <c r="S10" s="15"/>
+      <c r="T10" s="15"/>
+      <c r="U10" s="15"/>
+      <c r="V10" s="15">
+        <f t="shared" si="0"/>
+        <v>0.24</v>
+      </c>
+      <c r="W10" s="15"/>
+      <c r="Y10" s="6"/>
+    </row>
+    <row r="11" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
+      <c r="A11" s="20"/>
+      <c r="B11" s="20"/>
+      <c r="C11" s="20"/>
+      <c r="D11" s="20"/>
+      <c r="E11" s="20"/>
+      <c r="F11" s="20"/>
+      <c r="G11" s="20"/>
+      <c r="H11" s="20"/>
+      <c r="I11" s="20"/>
+      <c r="J11" s="20"/>
+      <c r="K11" s="20"/>
+      <c r="L11" s="20"/>
+      <c r="M11" s="20"/>
+      <c r="N11" s="20"/>
+      <c r="O11" s="20"/>
+      <c r="P11" s="20"/>
+      <c r="Q11" s="20"/>
+      <c r="R11" s="20"/>
+      <c r="S11" s="20"/>
+      <c r="T11" s="20"/>
+      <c r="U11" s="20"/>
+      <c r="V11" s="20"/>
+      <c r="W11" s="20"/>
+      <c r="Y11" s="22"/>
+    </row>
+    <row r="12" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A12" s="15"/>
+      <c r="B12" s="15"/>
+      <c r="C12" s="15" t="s">
+        <v>31</v>
+      </c>
+      <c r="D12" s="15"/>
+      <c r="E12" s="15"/>
+      <c r="F12" s="23"/>
+      <c r="G12" s="15"/>
+      <c r="H12" s="15"/>
+      <c r="I12" s="15"/>
+      <c r="J12" s="15"/>
+      <c r="K12" s="15"/>
+      <c r="L12" s="15"/>
+      <c r="M12" s="15"/>
+      <c r="N12" s="15"/>
+      <c r="O12" s="15"/>
+      <c r="P12" s="15">
+        <v>1</v>
+      </c>
+      <c r="Q12" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="R12" s="15"/>
+      <c r="S12" s="15"/>
+      <c r="T12" s="15"/>
+      <c r="U12" s="15"/>
+      <c r="V12" s="15">
         <f t="shared" si="0"/>
         <v>0.1</v>
       </c>
-      <c r="U7" s="14"/>
-      <c r="W7" s="29"/>
+      <c r="W12" s="23"/>
+      <c r="Y12" s="6"/>
     </row>
-    <row r="8" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A8" s="14"/>
-      <c r="B8" s="14"/>
-      <c r="C8" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="D8" s="14"/>
-      <c r="E8" s="14"/>
-      <c r="F8" s="14">
+    <row r="13" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
+      <c r="A13" s="20"/>
+      <c r="B13" s="20"/>
+      <c r="C13" s="20"/>
+      <c r="D13" s="20"/>
+      <c r="E13" s="20"/>
+      <c r="F13" s="20"/>
+      <c r="G13" s="20"/>
+      <c r="H13" s="20"/>
+      <c r="I13" s="20"/>
+      <c r="J13" s="20"/>
+      <c r="K13" s="20"/>
+      <c r="L13" s="20"/>
+      <c r="M13" s="20"/>
+      <c r="N13" s="20"/>
+      <c r="O13" s="20"/>
+      <c r="P13" s="20"/>
+      <c r="Q13" s="20"/>
+      <c r="R13" s="20"/>
+      <c r="S13" s="20"/>
+      <c r="T13" s="20"/>
+      <c r="U13" s="20"/>
+      <c r="V13" s="20"/>
+      <c r="W13" s="20"/>
+      <c r="Y13" s="22"/>
+    </row>
+    <row r="14" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A14" s="15"/>
+      <c r="B14" s="15"/>
+      <c r="C14" s="15" t="s">
+        <v>32</v>
+      </c>
+      <c r="D14" s="15"/>
+      <c r="E14" s="15"/>
+      <c r="F14" s="15"/>
+      <c r="G14" s="15"/>
+      <c r="H14" s="15"/>
+      <c r="I14" s="15"/>
+      <c r="J14" s="24">
+        <v>1</v>
+      </c>
+      <c r="K14" s="24">
+        <v>0.08</v>
+      </c>
+      <c r="L14" s="15"/>
+      <c r="M14" s="15"/>
+      <c r="N14" s="15"/>
+      <c r="O14" s="15"/>
+      <c r="P14" s="15">
+        <v>1</v>
+      </c>
+      <c r="Q14" s="15">
+        <v>0.1</v>
+      </c>
+      <c r="R14" s="15"/>
+      <c r="S14" s="15"/>
+      <c r="T14" s="15"/>
+      <c r="U14" s="15"/>
+      <c r="V14" s="15">
+        <f t="shared" ref="V14:V16" si="1">D14*E14+F14*G14+H14*I14+J14*K14+L14*M14+N14*O14+P14*Q14+R14*S14+T14*U14</f>
+        <v>0.18</v>
+      </c>
+      <c r="W14" s="15"/>
+      <c r="Y14" s="6"/>
+    </row>
+    <row r="15" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A15" s="15"/>
+      <c r="B15" s="15"/>
+      <c r="C15" s="15" t="s">
+        <v>33</v>
+      </c>
+      <c r="D15" s="15"/>
+      <c r="E15" s="15"/>
+      <c r="F15" s="15"/>
+      <c r="G15" s="15"/>
+      <c r="H15" s="15"/>
+      <c r="I15" s="15"/>
+      <c r="J15" s="15">
         <v>2</v>
       </c>
-      <c r="G8" s="14">
-        <v>0.05</v>
-      </c>
-      <c r="H8" s="14"/>
-      <c r="I8" s="14"/>
-      <c r="J8" s="14"/>
-      <c r="K8" s="14"/>
-      <c r="L8" s="14"/>
-      <c r="M8" s="14"/>
-      <c r="N8" s="14"/>
-      <c r="O8" s="14"/>
-      <c r="P8" s="14"/>
-      <c r="Q8" s="14"/>
-      <c r="R8" s="14"/>
-      <c r="S8" s="14"/>
-      <c r="T8" s="14">
-        <f t="shared" si="0"/>
-        <v>0.1</v>
-      </c>
-      <c r="U8" s="14"/>
-      <c r="W8" s="6"/>
-    </row>
-    <row r="9" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A9" s="14"/>
-      <c r="B9" s="14"/>
-      <c r="C9" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="D9" s="14"/>
-      <c r="E9" s="14"/>
-      <c r="F9" s="14">
-        <v>1</v>
-      </c>
-      <c r="G9" s="14">
-        <v>0.05</v>
-      </c>
-      <c r="H9" s="14"/>
-      <c r="I9" s="14"/>
-      <c r="J9" s="14"/>
-      <c r="K9" s="14"/>
-      <c r="L9" s="14"/>
-      <c r="M9" s="14"/>
-      <c r="N9" s="14"/>
-      <c r="O9" s="14"/>
-      <c r="P9" s="14"/>
-      <c r="Q9" s="14"/>
-      <c r="R9" s="14"/>
-      <c r="S9" s="14"/>
-      <c r="T9" s="14">
-        <f t="shared" si="0"/>
-        <v>0.05</v>
-      </c>
-      <c r="U9" s="14"/>
-      <c r="W9" s="6"/>
-    </row>
-    <row r="10" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A10" s="14"/>
-      <c r="B10" s="14"/>
-      <c r="C10" s="14" t="s">
-        <v>28</v>
-      </c>
-      <c r="D10" s="14"/>
-      <c r="E10" s="14"/>
-      <c r="F10" s="14"/>
-      <c r="G10" s="14"/>
-      <c r="H10" s="14">
-        <v>2</v>
-      </c>
-      <c r="I10" s="14">
+      <c r="K15" s="15">
         <v>0.08</v>
       </c>
-      <c r="J10" s="14">
-        <v>1</v>
-      </c>
-      <c r="K10" s="14">
-        <v>0.08</v>
-      </c>
-      <c r="L10" s="14"/>
-      <c r="M10" s="14"/>
-      <c r="N10" s="14"/>
-      <c r="O10" s="14"/>
-      <c r="P10" s="14"/>
-      <c r="Q10" s="14"/>
-      <c r="R10" s="14"/>
-      <c r="S10" s="14"/>
-      <c r="T10" s="14">
-        <f t="shared" si="0"/>
-        <v>0.24</v>
-      </c>
-      <c r="U10" s="14"/>
-      <c r="W10" s="6"/>
-    </row>
-    <row r="11" s="3" customFormat="1" ht="15" customHeight="1" spans="1:23">
-      <c r="A11" s="18"/>
-      <c r="B11" s="18"/>
-      <c r="C11" s="18"/>
-      <c r="D11" s="18"/>
-      <c r="E11" s="18"/>
-      <c r="F11" s="18"/>
-      <c r="G11" s="18"/>
-      <c r="H11" s="18"/>
-      <c r="I11" s="18"/>
-      <c r="J11" s="18"/>
-      <c r="K11" s="18"/>
-      <c r="L11" s="18"/>
-      <c r="M11" s="18"/>
-      <c r="N11" s="18"/>
-      <c r="O11" s="18"/>
-      <c r="P11" s="18"/>
-      <c r="Q11" s="18"/>
-      <c r="R11" s="18"/>
-      <c r="S11" s="18"/>
-      <c r="T11" s="18"/>
-      <c r="U11" s="18"/>
-      <c r="W11" s="31"/>
-    </row>
-    <row r="12" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A12" s="14"/>
-      <c r="B12" s="14"/>
-      <c r="C12" s="14" t="s">
-        <v>29</v>
-      </c>
-      <c r="D12" s="14"/>
-      <c r="E12" s="14"/>
-      <c r="F12" s="19"/>
-      <c r="G12" s="14"/>
-      <c r="H12" s="14"/>
-      <c r="I12" s="14"/>
-      <c r="J12" s="14"/>
-      <c r="K12" s="14"/>
-      <c r="L12" s="14"/>
-      <c r="M12" s="14"/>
-      <c r="N12" s="14">
-        <v>1</v>
-      </c>
-      <c r="O12" s="14">
-        <v>0.1</v>
-      </c>
-      <c r="P12" s="14"/>
-      <c r="Q12" s="14"/>
-      <c r="R12" s="14"/>
-      <c r="S12" s="14"/>
-      <c r="T12" s="14">
-        <f t="shared" ref="T12:T16" si="1">D12*E12+F12*G12+H12*I12+J12*K12+L12*M12+N12*O12+P12*Q12+R12*S12</f>
-        <v>0.1</v>
-      </c>
-      <c r="U12" s="19"/>
-      <c r="W12" s="6"/>
-    </row>
-    <row r="13" s="3" customFormat="1" ht="15" customHeight="1" spans="1:23">
-      <c r="A13" s="18"/>
-      <c r="B13" s="18"/>
-      <c r="C13" s="18"/>
-      <c r="D13" s="18"/>
-      <c r="E13" s="18"/>
-      <c r="F13" s="18"/>
-      <c r="G13" s="18"/>
-      <c r="H13" s="18"/>
-      <c r="I13" s="18"/>
-      <c r="J13" s="18"/>
-      <c r="K13" s="18"/>
-      <c r="L13" s="18"/>
-      <c r="M13" s="18"/>
-      <c r="N13" s="18"/>
-      <c r="O13" s="18"/>
-      <c r="P13" s="18"/>
-      <c r="Q13" s="18"/>
-      <c r="R13" s="18"/>
-      <c r="S13" s="18"/>
-      <c r="T13" s="18"/>
-      <c r="U13" s="18"/>
-      <c r="W13" s="31"/>
-    </row>
-    <row r="14" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A14" s="14"/>
-      <c r="B14" s="14"/>
-      <c r="C14" s="14" t="s">
-        <v>30</v>
-      </c>
-      <c r="D14" s="14"/>
-      <c r="E14" s="14"/>
-      <c r="F14" s="14"/>
-      <c r="G14" s="14"/>
-      <c r="H14" s="20">
-        <v>1</v>
-      </c>
-      <c r="I14" s="20">
-        <v>0.08</v>
-      </c>
-      <c r="J14" s="14"/>
-      <c r="K14" s="14"/>
-      <c r="L14" s="14"/>
-      <c r="M14" s="14"/>
-      <c r="N14" s="14">
-        <v>1</v>
-      </c>
-      <c r="O14" s="14">
-        <v>0.1</v>
-      </c>
-      <c r="P14" s="14"/>
-      <c r="Q14" s="14"/>
-      <c r="R14" s="14"/>
-      <c r="S14" s="14"/>
-      <c r="T14" s="14">
-        <f t="shared" si="1"/>
-        <v>0.18</v>
-      </c>
-      <c r="U14" s="14"/>
-      <c r="W14" s="6"/>
-    </row>
-    <row r="15" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A15" s="14"/>
-      <c r="B15" s="14"/>
-      <c r="C15" s="14" t="s">
-        <v>31</v>
-      </c>
-      <c r="D15" s="14"/>
-      <c r="E15" s="14"/>
-      <c r="F15" s="14"/>
-      <c r="G15" s="14"/>
-      <c r="H15" s="14">
-        <v>2</v>
-      </c>
-      <c r="I15" s="14">
-        <v>0.08</v>
-      </c>
-      <c r="J15" s="14"/>
-      <c r="K15" s="14"/>
-      <c r="L15" s="14"/>
-      <c r="M15" s="14"/>
-      <c r="N15" s="14"/>
-      <c r="O15" s="14"/>
-      <c r="P15" s="14"/>
-      <c r="Q15" s="14"/>
-      <c r="R15" s="14"/>
-      <c r="S15" s="14"/>
-      <c r="T15" s="14">
+      <c r="L15" s="15"/>
+      <c r="M15" s="15"/>
+      <c r="N15" s="15"/>
+      <c r="O15" s="15"/>
+      <c r="P15" s="15"/>
+      <c r="Q15" s="15"/>
+      <c r="R15" s="15"/>
+      <c r="S15" s="15"/>
+      <c r="T15" s="15"/>
+      <c r="U15" s="15"/>
+      <c r="V15" s="15">
         <f t="shared" si="1"/>
         <v>0.16</v>
       </c>
-      <c r="U15" s="14"/>
-      <c r="W15" s="6"/>
+      <c r="W15" s="15"/>
+      <c r="Y15" s="6"/>
     </row>
-    <row r="16" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A16" s="14"/>
-      <c r="B16" s="14"/>
-      <c r="C16" s="14" t="s">
-        <v>32</v>
-      </c>
-      <c r="D16" s="14"/>
-      <c r="E16" s="14"/>
-      <c r="F16" s="14"/>
-      <c r="G16" s="14"/>
-      <c r="H16" s="20">
+    <row r="16" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A16" s="15"/>
+      <c r="B16" s="15"/>
+      <c r="C16" s="15" t="s">
+        <v>34</v>
+      </c>
+      <c r="D16" s="15"/>
+      <c r="E16" s="15"/>
+      <c r="F16" s="15"/>
+      <c r="G16" s="15"/>
+      <c r="H16" s="15"/>
+      <c r="I16" s="15"/>
+      <c r="J16" s="24">
         <v>1</v>
       </c>
-      <c r="I16" s="20">
+      <c r="K16" s="24">
         <v>0.08</v>
       </c>
-      <c r="J16" s="14"/>
-      <c r="K16" s="14"/>
-      <c r="L16" s="14"/>
-      <c r="M16" s="14"/>
-      <c r="N16" s="14"/>
-      <c r="O16" s="14"/>
-      <c r="P16" s="14"/>
-      <c r="Q16" s="14"/>
-      <c r="R16" s="14"/>
-      <c r="S16" s="14"/>
-      <c r="T16" s="14">
+      <c r="L16" s="15"/>
+      <c r="M16" s="15"/>
+      <c r="N16" s="15"/>
+      <c r="O16" s="15"/>
+      <c r="P16" s="15"/>
+      <c r="Q16" s="15"/>
+      <c r="R16" s="15"/>
+      <c r="S16" s="15"/>
+      <c r="T16" s="15"/>
+      <c r="U16" s="15"/>
+      <c r="V16" s="15">
         <f t="shared" si="1"/>
         <v>0.08</v>
       </c>
-      <c r="U16" s="14"/>
-      <c r="W16" s="6"/>
+      <c r="W16" s="15"/>
+      <c r="Y16" s="6"/>
     </row>
-    <row r="17" s="4" customFormat="1" ht="20" customHeight="1" spans="1:23">
-      <c r="A17" s="21"/>
-      <c r="B17" s="21"/>
-      <c r="C17" s="21"/>
-      <c r="D17" s="21"/>
-      <c r="E17" s="21"/>
-      <c r="F17" s="21"/>
-      <c r="G17" s="21"/>
-      <c r="H17" s="21"/>
-      <c r="I17" s="21"/>
-      <c r="J17" s="21"/>
-      <c r="K17" s="21"/>
-      <c r="L17" s="21"/>
-      <c r="M17" s="21"/>
-      <c r="N17" s="21"/>
-      <c r="O17" s="21"/>
-      <c r="P17" s="21"/>
-      <c r="Q17" s="21"/>
-      <c r="R17" s="21"/>
-      <c r="S17" s="21"/>
-      <c r="T17" s="21"/>
-      <c r="U17" s="21"/>
-      <c r="W17" s="32"/>
+    <row r="17" s="4" customFormat="1" ht="20" customHeight="1" spans="1:25">
+      <c r="A17" s="25"/>
+      <c r="B17" s="25"/>
+      <c r="C17" s="25"/>
+      <c r="D17" s="25"/>
+      <c r="E17" s="25"/>
+      <c r="F17" s="25"/>
+      <c r="G17" s="25"/>
+      <c r="H17" s="25"/>
+      <c r="I17" s="25"/>
+      <c r="J17" s="25"/>
+      <c r="K17" s="25"/>
+      <c r="L17" s="25"/>
+      <c r="M17" s="25"/>
+      <c r="N17" s="25"/>
+      <c r="O17" s="25"/>
+      <c r="P17" s="25"/>
+      <c r="Q17" s="25"/>
+      <c r="R17" s="25"/>
+      <c r="S17" s="25"/>
+      <c r="T17" s="25"/>
+      <c r="U17" s="25"/>
+      <c r="V17" s="25"/>
+      <c r="W17" s="25"/>
+      <c r="Y17" s="26"/>
     </row>
-    <row r="18" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A18" s="14"/>
-      <c r="B18" s="22"/>
-      <c r="C18" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D18" s="13"/>
-      <c r="E18" s="14"/>
-      <c r="F18" s="14">
+    <row r="18" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A18" s="15"/>
+      <c r="B18" s="13"/>
+      <c r="C18" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D18" s="14"/>
+      <c r="E18" s="15"/>
+      <c r="F18" s="15">
         <v>2</v>
       </c>
-      <c r="G18" s="14">
+      <c r="G18" s="15">
         <v>0.15</v>
       </c>
-      <c r="H18" s="14"/>
-      <c r="I18" s="14"/>
-      <c r="J18" s="14"/>
-      <c r="K18" s="14"/>
-      <c r="L18" s="14"/>
-      <c r="M18" s="14"/>
-      <c r="N18" s="14"/>
-      <c r="O18" s="14"/>
-      <c r="P18" s="14"/>
-      <c r="Q18" s="14"/>
-      <c r="R18" s="14"/>
-      <c r="S18" s="14"/>
-      <c r="T18" s="14">
-        <f t="shared" ref="T18:T22" si="2">D18*E18+F18*G18+H18*I18+J18*K18+L18*M18+N18*O18+P18*Q18+R18*S18</f>
+      <c r="H18" s="15"/>
+      <c r="I18" s="15"/>
+      <c r="J18" s="15"/>
+      <c r="K18" s="15"/>
+      <c r="L18" s="15"/>
+      <c r="M18" s="15"/>
+      <c r="N18" s="15"/>
+      <c r="O18" s="15"/>
+      <c r="P18" s="15"/>
+      <c r="Q18" s="15"/>
+      <c r="R18" s="15"/>
+      <c r="S18" s="15"/>
+      <c r="T18" s="15"/>
+      <c r="U18" s="15"/>
+      <c r="V18" s="15">
+        <f>D18*E18+F18*G18+H18*I18+J18*K18+L18*M18+N18*O18+P18*Q18+R18*S18+T18*U18</f>
         <v>0.3</v>
       </c>
-      <c r="U18" s="14"/>
-      <c r="W18" s="6"/>
+      <c r="W18" s="15"/>
+      <c r="Y18" s="6"/>
     </row>
-    <row r="19" s="3" customFormat="1" ht="15" customHeight="1" spans="1:23">
-      <c r="A19" s="18"/>
-      <c r="B19" s="23"/>
-      <c r="C19" s="16"/>
-      <c r="D19" s="17"/>
-      <c r="E19" s="18"/>
-      <c r="F19" s="18"/>
-      <c r="G19" s="18"/>
-      <c r="H19" s="18"/>
-      <c r="I19" s="18"/>
-      <c r="J19" s="18"/>
-      <c r="K19" s="18"/>
-      <c r="L19" s="18"/>
-      <c r="M19" s="18"/>
-      <c r="N19" s="18"/>
-      <c r="O19" s="18"/>
-      <c r="P19" s="18"/>
-      <c r="Q19" s="18"/>
-      <c r="R19" s="18"/>
-      <c r="S19" s="18"/>
-      <c r="T19" s="18"/>
-      <c r="U19" s="18"/>
-      <c r="W19" s="31"/>
+    <row r="19" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
+      <c r="A19" s="20"/>
+      <c r="B19" s="18"/>
+      <c r="C19" s="18"/>
+      <c r="D19" s="19"/>
+      <c r="E19" s="20"/>
+      <c r="F19" s="20"/>
+      <c r="G19" s="20"/>
+      <c r="H19" s="20"/>
+      <c r="I19" s="20"/>
+      <c r="J19" s="20"/>
+      <c r="K19" s="20"/>
+      <c r="L19" s="20"/>
+      <c r="M19" s="20"/>
+      <c r="N19" s="20"/>
+      <c r="O19" s="20"/>
+      <c r="P19" s="20"/>
+      <c r="Q19" s="20"/>
+      <c r="R19" s="20"/>
+      <c r="S19" s="20"/>
+      <c r="T19" s="20"/>
+      <c r="U19" s="20"/>
+      <c r="V19" s="20"/>
+      <c r="W19" s="20"/>
+      <c r="Y19" s="22"/>
     </row>
-    <row r="20" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A20" s="14"/>
-      <c r="B20" s="14"/>
-      <c r="C20" s="14" t="s">
-        <v>27</v>
-      </c>
-      <c r="D20" s="14">
+    <row r="20" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A20" s="15"/>
+      <c r="B20" s="15"/>
+      <c r="C20" s="15" t="s">
+        <v>29</v>
+      </c>
+      <c r="D20" s="15">
         <v>3</v>
       </c>
-      <c r="E20" s="14">
+      <c r="E20" s="15">
         <v>0.12</v>
       </c>
-      <c r="F20" s="14">
+      <c r="F20" s="15">
         <v>2</v>
       </c>
-      <c r="G20" s="14">
+      <c r="G20" s="15">
         <v>0.05</v>
       </c>
-      <c r="H20" s="14"/>
-      <c r="I20" s="14"/>
-      <c r="J20" s="14"/>
-      <c r="K20" s="14"/>
-      <c r="L20" s="14"/>
-      <c r="M20" s="14"/>
-      <c r="N20" s="14">
+      <c r="H20" s="15"/>
+      <c r="I20" s="15"/>
+      <c r="J20" s="15"/>
+      <c r="K20" s="15"/>
+      <c r="L20" s="15"/>
+      <c r="M20" s="15"/>
+      <c r="N20" s="15"/>
+      <c r="O20" s="15"/>
+      <c r="P20" s="15">
         <v>1</v>
       </c>
-      <c r="O20" s="14">
+      <c r="Q20" s="15">
         <v>0.1</v>
       </c>
-      <c r="P20" s="14">
+      <c r="R20" s="15">
         <v>2</v>
       </c>
-      <c r="Q20" s="14">
+      <c r="S20" s="15">
         <v>0.1</v>
       </c>
-      <c r="R20" s="14"/>
-      <c r="S20" s="14"/>
-      <c r="T20" s="14">
-        <f t="shared" si="2"/>
+      <c r="T20" s="15"/>
+      <c r="U20" s="15"/>
+      <c r="V20" s="15">
+        <f t="shared" ref="V20:V24" si="2">D20*E20+F20*G20+H20*I20+J20*K20+L20*M20+N20*O20+P20*Q20+R20*S20+T20*U20</f>
         <v>0.76</v>
       </c>
-      <c r="U20" s="14"/>
-      <c r="W20" s="6"/>
+      <c r="W20" s="15"/>
+      <c r="Y20" s="6"/>
     </row>
-    <row r="21" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A21" s="14"/>
-      <c r="B21" s="14"/>
-      <c r="C21" s="14" t="s">
-        <v>26</v>
-      </c>
-      <c r="D21" s="14">
+    <row r="21" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A21" s="15"/>
+      <c r="B21" s="15"/>
+      <c r="C21" s="15" t="s">
+        <v>28</v>
+      </c>
+      <c r="D21" s="15">
         <v>2</v>
       </c>
-      <c r="E21" s="14">
+      <c r="E21" s="15">
         <v>0.12</v>
       </c>
-      <c r="F21" s="14"/>
-      <c r="G21" s="14"/>
-      <c r="H21" s="14"/>
-      <c r="I21" s="14"/>
-      <c r="J21" s="14">
+      <c r="F21" s="15"/>
+      <c r="G21" s="15"/>
+      <c r="H21" s="15"/>
+      <c r="I21" s="15"/>
+      <c r="J21" s="15"/>
+      <c r="K21" s="15"/>
+      <c r="L21" s="15">
         <v>1</v>
       </c>
-      <c r="K21" s="14">
+      <c r="M21" s="15">
         <v>0.08</v>
       </c>
-      <c r="L21" s="14"/>
-      <c r="M21" s="14"/>
-      <c r="N21" s="14">
+      <c r="N21" s="15"/>
+      <c r="O21" s="15"/>
+      <c r="P21" s="15">
         <v>1</v>
       </c>
-      <c r="O21" s="14">
+      <c r="Q21" s="15">
         <v>0.1</v>
       </c>
-      <c r="P21" s="14">
+      <c r="R21" s="15">
         <v>3</v>
       </c>
-      <c r="Q21" s="14">
+      <c r="S21" s="15">
         <v>0.1</v>
       </c>
-      <c r="R21" s="14"/>
-      <c r="S21" s="14"/>
-      <c r="T21" s="14">
+      <c r="T21" s="15"/>
+      <c r="U21" s="15"/>
+      <c r="V21" s="15">
         <f t="shared" si="2"/>
         <v>0.72</v>
       </c>
-      <c r="U21" s="14"/>
-      <c r="W21" s="6"/>
+      <c r="W21" s="15"/>
+      <c r="Y21" s="6"/>
     </row>
-    <row r="22" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A22" s="14"/>
-      <c r="B22" s="14"/>
-      <c r="C22" s="14" t="s">
-        <v>33</v>
-      </c>
-      <c r="D22" s="14">
+    <row r="22" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A22" s="15"/>
+      <c r="B22" s="15"/>
+      <c r="C22" s="15" t="s">
+        <v>35</v>
+      </c>
+      <c r="D22" s="15">
         <v>1</v>
       </c>
-      <c r="E22" s="14">
+      <c r="E22" s="15">
         <v>0.12</v>
       </c>
-      <c r="F22" s="14"/>
-      <c r="G22" s="14"/>
-      <c r="H22" s="14"/>
-      <c r="I22" s="14"/>
-      <c r="J22" s="14"/>
-      <c r="K22" s="14"/>
-      <c r="L22" s="14"/>
-      <c r="M22" s="14"/>
-      <c r="N22" s="14">
+      <c r="F22" s="15"/>
+      <c r="G22" s="15"/>
+      <c r="H22" s="15"/>
+      <c r="I22" s="15"/>
+      <c r="J22" s="15"/>
+      <c r="K22" s="15"/>
+      <c r="L22" s="15"/>
+      <c r="M22" s="15"/>
+      <c r="N22" s="15"/>
+      <c r="O22" s="15"/>
+      <c r="P22" s="15">
         <v>1</v>
       </c>
-      <c r="O22" s="14">
+      <c r="Q22" s="15">
         <v>0.1</v>
       </c>
-      <c r="P22" s="14">
+      <c r="R22" s="15">
         <v>2</v>
       </c>
-      <c r="Q22" s="14">
+      <c r="S22" s="15">
         <v>0.1</v>
       </c>
-      <c r="R22" s="14"/>
-      <c r="S22" s="14"/>
-      <c r="T22" s="14">
+      <c r="T22" s="15"/>
+      <c r="U22" s="15"/>
+      <c r="V22" s="15">
         <f t="shared" si="2"/>
         <v>0.42</v>
       </c>
-      <c r="U22" s="14"/>
-      <c r="W22" s="6"/>
+      <c r="W22" s="15"/>
+      <c r="Y22" s="6"/>
     </row>
-    <row r="23" s="3" customFormat="1" ht="15" customHeight="1" spans="1:23">
-      <c r="A23" s="18"/>
-      <c r="B23" s="18"/>
-      <c r="C23" s="18"/>
-      <c r="D23" s="18"/>
-      <c r="E23" s="18"/>
-      <c r="F23" s="18"/>
-      <c r="G23" s="18"/>
-      <c r="H23" s="18"/>
-      <c r="I23" s="18"/>
-      <c r="J23" s="18"/>
-      <c r="K23" s="18"/>
-      <c r="L23" s="18"/>
-      <c r="M23" s="18"/>
-      <c r="N23" s="18"/>
-      <c r="O23" s="18"/>
-      <c r="P23" s="18"/>
-      <c r="Q23" s="18"/>
-      <c r="R23" s="18"/>
-      <c r="S23" s="18"/>
-      <c r="T23" s="18"/>
-      <c r="U23" s="18"/>
-      <c r="W23" s="31"/>
+    <row r="23" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
+      <c r="A23" s="20"/>
+      <c r="B23" s="20"/>
+      <c r="C23" s="20"/>
+      <c r="D23" s="20"/>
+      <c r="E23" s="20"/>
+      <c r="F23" s="20"/>
+      <c r="G23" s="20"/>
+      <c r="H23" s="20"/>
+      <c r="I23" s="20"/>
+      <c r="J23" s="20"/>
+      <c r="K23" s="20"/>
+      <c r="L23" s="20"/>
+      <c r="M23" s="20"/>
+      <c r="N23" s="20"/>
+      <c r="O23" s="20"/>
+      <c r="P23" s="20"/>
+      <c r="Q23" s="20"/>
+      <c r="R23" s="20"/>
+      <c r="S23" s="20"/>
+      <c r="T23" s="20"/>
+      <c r="U23" s="20"/>
+      <c r="V23" s="20"/>
+      <c r="W23" s="20"/>
+      <c r="Y23" s="22"/>
     </row>
-    <row r="24" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A24" s="14"/>
-      <c r="B24" s="14"/>
-      <c r="C24" s="14" t="s">
-        <v>34</v>
-      </c>
-      <c r="D24" s="14">
+    <row r="24" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A24" s="15"/>
+      <c r="B24" s="15"/>
+      <c r="C24" s="15" t="s">
+        <v>36</v>
+      </c>
+      <c r="D24" s="15">
         <v>3</v>
       </c>
-      <c r="E24" s="14">
+      <c r="E24" s="15">
         <v>0.12</v>
       </c>
-      <c r="F24" s="19"/>
-      <c r="G24" s="14"/>
-      <c r="H24" s="14"/>
-      <c r="I24" s="14"/>
-      <c r="J24" s="14">
+      <c r="F24" s="23"/>
+      <c r="G24" s="15"/>
+      <c r="H24" s="15"/>
+      <c r="I24" s="15"/>
+      <c r="J24" s="15"/>
+      <c r="K24" s="15"/>
+      <c r="L24" s="15">
         <v>8</v>
       </c>
-      <c r="K24" s="14">
+      <c r="M24" s="15">
         <v>0.08</v>
       </c>
-      <c r="L24" s="14"/>
-      <c r="M24" s="14"/>
-      <c r="N24" s="14"/>
-      <c r="O24" s="14"/>
-      <c r="P24" s="14"/>
-      <c r="Q24" s="14"/>
-      <c r="R24" s="14"/>
-      <c r="S24" s="14"/>
-      <c r="T24" s="14">
-        <f t="shared" ref="T24:T27" si="3">D24*E24+F24*G24+H24*I24+J24*K24+L24*M24+N24*O24+P24*Q24+R24*S24</f>
+      <c r="N24" s="15"/>
+      <c r="O24" s="15"/>
+      <c r="P24" s="15"/>
+      <c r="Q24" s="15"/>
+      <c r="R24" s="15"/>
+      <c r="S24" s="15"/>
+      <c r="T24" s="15"/>
+      <c r="U24" s="15"/>
+      <c r="V24" s="15">
+        <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="U24" s="14"/>
-      <c r="W24" s="6"/>
+      <c r="W24" s="15"/>
+      <c r="Y24" s="6"/>
     </row>
-    <row r="25" s="3" customFormat="1" ht="15" customHeight="1" spans="1:23">
-      <c r="A25" s="18"/>
-      <c r="B25" s="18"/>
-      <c r="C25" s="18"/>
-      <c r="D25" s="18"/>
-      <c r="E25" s="18"/>
-      <c r="F25" s="18"/>
-      <c r="G25" s="18"/>
-      <c r="H25" s="18"/>
-      <c r="I25" s="18"/>
-      <c r="J25" s="18"/>
-      <c r="K25" s="18"/>
-      <c r="L25" s="18"/>
-      <c r="M25" s="18"/>
-      <c r="N25" s="18"/>
-      <c r="O25" s="18"/>
-      <c r="P25" s="18"/>
-      <c r="Q25" s="18"/>
-      <c r="R25" s="18"/>
-      <c r="S25" s="18"/>
-      <c r="T25" s="18"/>
-      <c r="U25" s="18"/>
-      <c r="W25" s="31"/>
+    <row r="25" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
+      <c r="A25" s="20"/>
+      <c r="B25" s="20"/>
+      <c r="C25" s="20"/>
+      <c r="D25" s="20"/>
+      <c r="E25" s="20"/>
+      <c r="F25" s="20"/>
+      <c r="G25" s="20"/>
+      <c r="H25" s="20"/>
+      <c r="I25" s="20"/>
+      <c r="J25" s="20"/>
+      <c r="K25" s="20"/>
+      <c r="L25" s="20"/>
+      <c r="M25" s="20"/>
+      <c r="N25" s="20"/>
+      <c r="O25" s="20"/>
+      <c r="P25" s="20"/>
+      <c r="Q25" s="20"/>
+      <c r="R25" s="20"/>
+      <c r="S25" s="20"/>
+      <c r="T25" s="20"/>
+      <c r="U25" s="20"/>
+      <c r="V25" s="20"/>
+      <c r="W25" s="20"/>
+      <c r="Y25" s="22"/>
     </row>
-    <row r="26" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A26" s="14"/>
-      <c r="B26" s="14"/>
-      <c r="C26" s="14" t="s">
-        <v>35</v>
-      </c>
-      <c r="D26" s="14"/>
-      <c r="E26" s="14"/>
-      <c r="F26" s="14"/>
-      <c r="G26" s="14"/>
-      <c r="H26" s="20">
+    <row r="26" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A26" s="15"/>
+      <c r="B26" s="15"/>
+      <c r="C26" s="15" t="s">
+        <v>37</v>
+      </c>
+      <c r="D26" s="15"/>
+      <c r="E26" s="15"/>
+      <c r="F26" s="15"/>
+      <c r="G26" s="15"/>
+      <c r="H26" s="15"/>
+      <c r="I26" s="15"/>
+      <c r="J26" s="24">
         <v>1</v>
       </c>
-      <c r="I26" s="20">
+      <c r="K26" s="24">
         <v>0.08</v>
       </c>
-      <c r="J26" s="14"/>
-      <c r="K26" s="14"/>
-      <c r="L26" s="14"/>
-      <c r="M26" s="14"/>
-      <c r="N26" s="14"/>
-      <c r="O26" s="14"/>
-      <c r="P26" s="14"/>
-      <c r="Q26" s="14"/>
-      <c r="R26" s="14"/>
-      <c r="S26" s="14"/>
-      <c r="T26" s="14">
-        <f t="shared" si="3"/>
+      <c r="L26" s="15"/>
+      <c r="M26" s="15"/>
+      <c r="N26" s="15"/>
+      <c r="O26" s="15"/>
+      <c r="P26" s="15"/>
+      <c r="Q26" s="15"/>
+      <c r="R26" s="15"/>
+      <c r="S26" s="15"/>
+      <c r="T26" s="15"/>
+      <c r="U26" s="15"/>
+      <c r="V26" s="15">
+        <f t="shared" ref="V26:V29" si="3">D26*E26+F26*G26+H26*I26+J26*K26+L26*M26+N26*O26+P26*Q26+R26*S26+T26*U26</f>
         <v>0.08</v>
       </c>
-      <c r="U26" s="14"/>
-      <c r="W26" s="6"/>
+      <c r="W26" s="15"/>
+      <c r="Y26" s="6"/>
     </row>
-    <row r="27" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A27" s="14"/>
-      <c r="B27" s="14"/>
-      <c r="C27" s="14" t="s">
-        <v>36</v>
-      </c>
-      <c r="D27" s="14"/>
-      <c r="E27" s="14"/>
-      <c r="F27" s="14"/>
-      <c r="G27" s="14"/>
-      <c r="H27" s="14">
+    <row r="27" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A27" s="15"/>
+      <c r="B27" s="15"/>
+      <c r="C27" s="15" t="s">
+        <v>38</v>
+      </c>
+      <c r="D27" s="15"/>
+      <c r="E27" s="15"/>
+      <c r="F27" s="15"/>
+      <c r="G27" s="15"/>
+      <c r="H27" s="15"/>
+      <c r="I27" s="15"/>
+      <c r="J27" s="15">
         <v>2</v>
       </c>
-      <c r="I27" s="14">
+      <c r="K27" s="15">
         <v>0.08</v>
       </c>
-      <c r="J27" s="14"/>
-      <c r="K27" s="14"/>
-      <c r="L27" s="14"/>
-      <c r="M27" s="14"/>
-      <c r="N27" s="14"/>
-      <c r="O27" s="14"/>
-      <c r="P27" s="14"/>
-      <c r="Q27" s="14"/>
-      <c r="R27" s="14"/>
-      <c r="S27" s="14"/>
-      <c r="T27" s="14">
+      <c r="L27" s="15"/>
+      <c r="M27" s="15"/>
+      <c r="N27" s="15"/>
+      <c r="O27" s="15"/>
+      <c r="P27" s="15"/>
+      <c r="Q27" s="15"/>
+      <c r="R27" s="15"/>
+      <c r="S27" s="15"/>
+      <c r="T27" s="15"/>
+      <c r="U27" s="15"/>
+      <c r="V27" s="15">
         <f t="shared" si="3"/>
         <v>0.16</v>
       </c>
-      <c r="U27" s="33"/>
-      <c r="W27" s="6"/>
+      <c r="W27" s="27"/>
+      <c r="Y27" s="6"/>
     </row>
-    <row r="28" s="3" customFormat="1" ht="15" customHeight="1" spans="1:23">
-      <c r="A28" s="18"/>
-      <c r="B28" s="18"/>
-      <c r="C28" s="18"/>
-      <c r="D28" s="18"/>
-      <c r="E28" s="18"/>
-      <c r="F28" s="18"/>
-      <c r="G28" s="18"/>
-      <c r="H28" s="18"/>
-      <c r="I28" s="18"/>
-      <c r="J28" s="18"/>
-      <c r="K28" s="18"/>
-      <c r="L28" s="18"/>
-      <c r="M28" s="18"/>
-      <c r="N28" s="18"/>
-      <c r="O28" s="18"/>
-      <c r="P28" s="18"/>
-      <c r="Q28" s="18"/>
-      <c r="R28" s="18"/>
-      <c r="S28" s="18"/>
-      <c r="T28" s="18"/>
-      <c r="U28" s="34"/>
-      <c r="W28" s="31"/>
+    <row r="28" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
+      <c r="A28" s="20"/>
+      <c r="B28" s="20"/>
+      <c r="C28" s="20"/>
+      <c r="D28" s="20"/>
+      <c r="E28" s="20"/>
+      <c r="F28" s="20"/>
+      <c r="G28" s="20"/>
+      <c r="H28" s="20"/>
+      <c r="I28" s="20"/>
+      <c r="J28" s="20"/>
+      <c r="K28" s="20"/>
+      <c r="L28" s="20"/>
+      <c r="M28" s="20"/>
+      <c r="N28" s="20"/>
+      <c r="O28" s="20"/>
+      <c r="P28" s="20"/>
+      <c r="Q28" s="20"/>
+      <c r="R28" s="20"/>
+      <c r="S28" s="20"/>
+      <c r="T28" s="20"/>
+      <c r="U28" s="20"/>
+      <c r="V28" s="20"/>
+      <c r="W28" s="28"/>
+      <c r="Y28" s="22"/>
     </row>
-    <row r="29" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A29" s="14"/>
-      <c r="B29" s="14"/>
-      <c r="C29" s="14" t="s">
-        <v>37</v>
-      </c>
-      <c r="D29" s="14">
+    <row r="29" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A29" s="15"/>
+      <c r="B29" s="15"/>
+      <c r="C29" s="15" t="s">
+        <v>39</v>
+      </c>
+      <c r="D29" s="15">
         <v>2</v>
       </c>
-      <c r="E29" s="14">
+      <c r="E29" s="15">
         <v>0.12</v>
       </c>
-      <c r="F29" s="14"/>
-      <c r="G29" s="14"/>
-      <c r="H29" s="20">
+      <c r="F29" s="15"/>
+      <c r="G29" s="15"/>
+      <c r="H29" s="15"/>
+      <c r="I29" s="15"/>
+      <c r="J29" s="24">
         <v>1</v>
       </c>
-      <c r="I29" s="20">
+      <c r="K29" s="24">
         <v>0.08</v>
       </c>
-      <c r="J29" s="14"/>
-      <c r="K29" s="14"/>
-      <c r="L29" s="14"/>
-      <c r="M29" s="14"/>
-      <c r="N29" s="14"/>
-      <c r="O29" s="14"/>
-      <c r="P29" s="19"/>
-      <c r="Q29" s="14"/>
-      <c r="R29" s="14"/>
-      <c r="S29" s="14"/>
-      <c r="T29" s="14">
-        <f t="shared" ref="T29:T35" si="4">D29*E29+F29*G29+H29*I29+J29*K29+L29*M29+N29*O29+P29*Q29+R29*S29</f>
+      <c r="L29" s="15"/>
+      <c r="M29" s="15"/>
+      <c r="N29" s="15"/>
+      <c r="O29" s="15"/>
+      <c r="P29" s="15"/>
+      <c r="Q29" s="15"/>
+      <c r="R29" s="23"/>
+      <c r="S29" s="15"/>
+      <c r="T29" s="15"/>
+      <c r="U29" s="15"/>
+      <c r="V29" s="15">
+        <f t="shared" si="3"/>
         <v>0.32</v>
       </c>
-      <c r="U29" s="14"/>
-      <c r="W29" s="6"/>
+      <c r="W29" s="15"/>
+      <c r="Y29" s="6"/>
     </row>
-    <row r="30" s="4" customFormat="1" ht="20" customHeight="1" spans="1:23">
-      <c r="A30" s="21"/>
-      <c r="B30" s="21"/>
-      <c r="C30" s="21"/>
-      <c r="D30" s="21"/>
-      <c r="E30" s="21"/>
-      <c r="F30" s="21"/>
-      <c r="G30" s="21"/>
-      <c r="H30" s="21"/>
-      <c r="I30" s="21"/>
-      <c r="J30" s="21"/>
-      <c r="K30" s="21"/>
-      <c r="L30" s="21"/>
-      <c r="M30" s="21"/>
-      <c r="N30" s="21"/>
-      <c r="O30" s="21"/>
-      <c r="P30" s="21"/>
-      <c r="Q30" s="21"/>
-      <c r="R30" s="21"/>
-      <c r="S30" s="21"/>
-      <c r="T30" s="21"/>
-      <c r="U30" s="21"/>
-      <c r="W30" s="32"/>
+    <row r="30" s="4" customFormat="1" ht="20" customHeight="1" spans="1:25">
+      <c r="A30" s="25"/>
+      <c r="B30" s="25"/>
+      <c r="C30" s="25"/>
+      <c r="D30" s="25"/>
+      <c r="E30" s="25"/>
+      <c r="F30" s="25"/>
+      <c r="G30" s="25"/>
+      <c r="H30" s="25"/>
+      <c r="I30" s="25"/>
+      <c r="J30" s="25"/>
+      <c r="K30" s="25"/>
+      <c r="L30" s="25"/>
+      <c r="M30" s="25"/>
+      <c r="N30" s="25"/>
+      <c r="O30" s="25"/>
+      <c r="P30" s="25"/>
+      <c r="Q30" s="25"/>
+      <c r="R30" s="25"/>
+      <c r="S30" s="25"/>
+      <c r="T30" s="25"/>
+      <c r="U30" s="25"/>
+      <c r="V30" s="25"/>
+      <c r="W30" s="25"/>
+      <c r="Y30" s="26"/>
     </row>
-    <row r="31" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A31" s="14"/>
-      <c r="B31" s="22"/>
-      <c r="C31" s="12" t="s">
-        <v>22</v>
-      </c>
-      <c r="D31" s="24"/>
-      <c r="E31" s="14"/>
-      <c r="F31" s="14">
+    <row r="31" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A31" s="15"/>
+      <c r="B31" s="13"/>
+      <c r="C31" s="13" t="s">
+        <v>24</v>
+      </c>
+      <c r="D31" s="29"/>
+      <c r="E31" s="15"/>
+      <c r="F31" s="15">
         <v>2</v>
       </c>
-      <c r="G31" s="14">
+      <c r="G31" s="15">
         <v>0.15</v>
       </c>
-      <c r="H31" s="14"/>
-      <c r="I31" s="14"/>
-      <c r="J31" s="14"/>
-      <c r="K31" s="14"/>
-      <c r="L31" s="14"/>
-      <c r="M31" s="14"/>
-      <c r="N31" s="14"/>
-      <c r="O31" s="14"/>
-      <c r="P31" s="14"/>
-      <c r="Q31" s="14"/>
-      <c r="R31" s="14"/>
-      <c r="S31" s="14"/>
-      <c r="T31" s="14">
-        <f t="shared" si="4"/>
+      <c r="H31" s="15"/>
+      <c r="I31" s="15"/>
+      <c r="J31" s="15"/>
+      <c r="K31" s="15"/>
+      <c r="L31" s="15"/>
+      <c r="M31" s="15"/>
+      <c r="N31" s="15"/>
+      <c r="O31" s="15"/>
+      <c r="P31" s="15"/>
+      <c r="Q31" s="15"/>
+      <c r="R31" s="15"/>
+      <c r="S31" s="15"/>
+      <c r="T31" s="15"/>
+      <c r="U31" s="15"/>
+      <c r="V31" s="15">
+        <f>D31*E31+F31*G31+H31*I31+J31*K31+L31*M31+N31*O31+P31*Q31+R31*S31+T31*U31</f>
         <v>0.3</v>
       </c>
-      <c r="U31" s="14"/>
-      <c r="W31" s="6"/>
+      <c r="W31" s="15"/>
+      <c r="Y31" s="6"/>
     </row>
-    <row r="32" s="3" customFormat="1" ht="15" customHeight="1" spans="1:23">
-      <c r="A32" s="18"/>
-      <c r="B32" s="23"/>
-      <c r="C32" s="16"/>
-      <c r="D32" s="17"/>
-      <c r="E32" s="18"/>
-      <c r="F32" s="18"/>
-      <c r="G32" s="18"/>
-      <c r="H32" s="18"/>
-      <c r="I32" s="18"/>
-      <c r="J32" s="18"/>
-      <c r="K32" s="18"/>
-      <c r="L32" s="18"/>
-      <c r="M32" s="18"/>
-      <c r="N32" s="18"/>
-      <c r="O32" s="18"/>
-      <c r="P32" s="18"/>
-      <c r="Q32" s="18"/>
-      <c r="R32" s="18"/>
-      <c r="S32" s="18"/>
-      <c r="T32" s="18"/>
-      <c r="U32" s="18"/>
-      <c r="W32" s="31"/>
+    <row r="32" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
+      <c r="A32" s="20"/>
+      <c r="B32" s="18"/>
+      <c r="C32" s="18"/>
+      <c r="D32" s="19"/>
+      <c r="E32" s="20"/>
+      <c r="F32" s="20"/>
+      <c r="G32" s="20"/>
+      <c r="H32" s="20"/>
+      <c r="I32" s="20"/>
+      <c r="J32" s="20"/>
+      <c r="K32" s="20"/>
+      <c r="L32" s="20"/>
+      <c r="M32" s="20"/>
+      <c r="N32" s="20"/>
+      <c r="O32" s="20"/>
+      <c r="P32" s="20"/>
+      <c r="Q32" s="20"/>
+      <c r="R32" s="20"/>
+      <c r="S32" s="20"/>
+      <c r="T32" s="20"/>
+      <c r="U32" s="20"/>
+      <c r="V32" s="20"/>
+      <c r="W32" s="20"/>
+      <c r="Y32" s="22"/>
     </row>
-    <row r="33" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A33" s="14"/>
-      <c r="B33" s="14"/>
-      <c r="C33" s="14" t="s">
-        <v>38</v>
-      </c>
-      <c r="D33" s="13"/>
-      <c r="E33" s="14"/>
-      <c r="F33" s="14"/>
-      <c r="G33" s="14"/>
-      <c r="H33" s="14"/>
-      <c r="I33" s="14"/>
-      <c r="J33" s="14">
+    <row r="33" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A33" s="15"/>
+      <c r="B33" s="15"/>
+      <c r="C33" s="15" t="s">
+        <v>40</v>
+      </c>
+      <c r="D33" s="14"/>
+      <c r="E33" s="15"/>
+      <c r="F33" s="15"/>
+      <c r="G33" s="15"/>
+      <c r="H33" s="15"/>
+      <c r="I33" s="15"/>
+      <c r="J33" s="15"/>
+      <c r="K33" s="15"/>
+      <c r="L33" s="15">
         <v>1</v>
       </c>
-      <c r="K33" s="14">
+      <c r="M33" s="15">
         <v>0.08</v>
       </c>
-      <c r="L33" s="14">
+      <c r="N33" s="15">
         <v>2</v>
       </c>
-      <c r="M33" s="14">
+      <c r="O33" s="15">
         <v>0.12</v>
       </c>
-      <c r="N33" s="14">
+      <c r="P33" s="15">
         <v>2</v>
       </c>
-      <c r="O33" s="14">
+      <c r="Q33" s="15">
         <v>0.1</v>
       </c>
-      <c r="P33" s="14">
+      <c r="R33" s="15">
         <v>5</v>
       </c>
-      <c r="Q33" s="14">
+      <c r="S33" s="15">
         <v>0.1</v>
       </c>
-      <c r="R33" s="14"/>
-      <c r="S33" s="14"/>
-      <c r="T33" s="14">
-        <f t="shared" si="4"/>
+      <c r="T33" s="15"/>
+      <c r="U33" s="15"/>
+      <c r="V33" s="15">
+        <f t="shared" ref="V33:V37" si="4">D33*E33+F33*G33+H33*I33+J33*K33+L33*M33+N33*O33+P33*Q33+R33*S33+T33*U33</f>
         <v>1.02</v>
       </c>
-      <c r="U33" s="14"/>
-      <c r="W33" s="6"/>
+      <c r="W33" s="15"/>
+      <c r="Y33" s="6"/>
     </row>
-    <row r="34" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A34" s="14"/>
-      <c r="B34" s="14"/>
-      <c r="C34" s="14" t="s">
-        <v>23</v>
-      </c>
-      <c r="D34" s="14"/>
-      <c r="E34" s="14"/>
-      <c r="F34" s="14">
+    <row r="34" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A34" s="15"/>
+      <c r="B34" s="15"/>
+      <c r="C34" s="15" t="s">
+        <v>25</v>
+      </c>
+      <c r="D34" s="15"/>
+      <c r="E34" s="15"/>
+      <c r="F34" s="15">
         <v>2</v>
       </c>
-      <c r="G34" s="14">
+      <c r="G34" s="15">
         <v>0.05</v>
       </c>
-      <c r="H34" s="14"/>
-      <c r="I34" s="14"/>
-      <c r="J34" s="14"/>
-      <c r="K34" s="14"/>
-      <c r="L34" s="14"/>
-      <c r="M34" s="14"/>
-      <c r="N34" s="14"/>
-      <c r="O34" s="14"/>
-      <c r="P34" s="14"/>
-      <c r="Q34" s="14"/>
-      <c r="R34" s="14"/>
-      <c r="S34" s="14"/>
-      <c r="T34" s="14">
+      <c r="H34" s="15"/>
+      <c r="I34" s="15"/>
+      <c r="J34" s="15"/>
+      <c r="K34" s="15"/>
+      <c r="L34" s="15"/>
+      <c r="M34" s="15"/>
+      <c r="N34" s="15"/>
+      <c r="O34" s="15"/>
+      <c r="P34" s="15"/>
+      <c r="Q34" s="15"/>
+      <c r="R34" s="15"/>
+      <c r="S34" s="15"/>
+      <c r="T34" s="15"/>
+      <c r="U34" s="15"/>
+      <c r="V34" s="15">
         <f t="shared" si="4"/>
         <v>0.1</v>
       </c>
-      <c r="U34" s="14"/>
-      <c r="W34" s="6"/>
+      <c r="W34" s="15"/>
+      <c r="Y34" s="6"/>
     </row>
-    <row r="35" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A35" s="14"/>
-      <c r="B35" s="14"/>
-      <c r="C35" s="14" t="s">
-        <v>39</v>
-      </c>
-      <c r="D35" s="14"/>
-      <c r="E35" s="14"/>
-      <c r="F35" s="14">
+    <row r="35" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A35" s="15"/>
+      <c r="B35" s="15"/>
+      <c r="C35" s="15" t="s">
+        <v>41</v>
+      </c>
+      <c r="D35" s="15"/>
+      <c r="E35" s="15"/>
+      <c r="F35" s="15">
         <v>4</v>
       </c>
-      <c r="G35" s="14">
+      <c r="G35" s="15">
         <v>0.05</v>
       </c>
-      <c r="H35" s="14"/>
-      <c r="I35" s="14"/>
-      <c r="J35" s="14"/>
-      <c r="K35" s="14"/>
-      <c r="L35" s="14"/>
-      <c r="M35" s="14"/>
-      <c r="N35" s="14"/>
-      <c r="O35" s="14"/>
-      <c r="P35" s="14"/>
-      <c r="Q35" s="14"/>
-      <c r="R35" s="14"/>
-      <c r="S35" s="14"/>
-      <c r="T35" s="14">
+      <c r="H35" s="15"/>
+      <c r="I35" s="15"/>
+      <c r="J35" s="15"/>
+      <c r="K35" s="15"/>
+      <c r="L35" s="15"/>
+      <c r="M35" s="15"/>
+      <c r="N35" s="15"/>
+      <c r="O35" s="15"/>
+      <c r="P35" s="15"/>
+      <c r="Q35" s="15"/>
+      <c r="R35" s="15"/>
+      <c r="S35" s="15"/>
+      <c r="T35" s="15"/>
+      <c r="U35" s="15"/>
+      <c r="V35" s="15">
         <f t="shared" si="4"/>
         <v>0.2</v>
       </c>
-      <c r="U35" s="14"/>
-      <c r="W35" s="6"/>
+      <c r="W35" s="15"/>
+      <c r="Y35" s="6"/>
     </row>
-    <row r="36" s="3" customFormat="1" ht="15" customHeight="1" spans="1:23">
-      <c r="A36" s="18"/>
-      <c r="B36" s="18"/>
-      <c r="C36" s="18"/>
-      <c r="D36" s="18"/>
-      <c r="E36" s="18"/>
-      <c r="F36" s="18"/>
-      <c r="G36" s="18"/>
-      <c r="H36" s="18"/>
-      <c r="I36" s="18"/>
-      <c r="J36" s="18"/>
-      <c r="K36" s="18"/>
-      <c r="L36" s="18"/>
-      <c r="M36" s="18"/>
-      <c r="N36" s="18"/>
-      <c r="O36" s="18"/>
-      <c r="P36" s="18"/>
-      <c r="Q36" s="18"/>
-      <c r="R36" s="18"/>
-      <c r="S36" s="18"/>
-      <c r="T36" s="18"/>
-      <c r="U36" s="18"/>
-      <c r="W36" s="31"/>
+    <row r="36" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
+      <c r="A36" s="20"/>
+      <c r="B36" s="20"/>
+      <c r="C36" s="20"/>
+      <c r="D36" s="20"/>
+      <c r="E36" s="20"/>
+      <c r="F36" s="20"/>
+      <c r="G36" s="20"/>
+      <c r="H36" s="20"/>
+      <c r="I36" s="20"/>
+      <c r="J36" s="20"/>
+      <c r="K36" s="20"/>
+      <c r="L36" s="20"/>
+      <c r="M36" s="20"/>
+      <c r="N36" s="20"/>
+      <c r="O36" s="20"/>
+      <c r="P36" s="20"/>
+      <c r="Q36" s="20"/>
+      <c r="R36" s="20"/>
+      <c r="S36" s="20"/>
+      <c r="T36" s="20"/>
+      <c r="U36" s="20"/>
+      <c r="V36" s="20"/>
+      <c r="W36" s="20"/>
+      <c r="Y36" s="22"/>
     </row>
-    <row r="37" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A37" s="14"/>
-      <c r="B37" s="14"/>
-      <c r="C37" s="14" t="s">
-        <v>40</v>
-      </c>
-      <c r="D37" s="14"/>
-      <c r="E37" s="14"/>
-      <c r="F37" s="14">
+    <row r="37" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A37" s="15"/>
+      <c r="B37" s="15"/>
+      <c r="C37" s="15" t="s">
+        <v>42</v>
+      </c>
+      <c r="D37" s="15"/>
+      <c r="E37" s="15"/>
+      <c r="F37" s="15">
         <v>1</v>
       </c>
-      <c r="G37" s="14">
+      <c r="G37" s="15">
         <v>0.05</v>
       </c>
-      <c r="H37" s="14"/>
-      <c r="I37" s="14"/>
-      <c r="J37" s="14">
+      <c r="H37" s="15"/>
+      <c r="I37" s="15"/>
+      <c r="J37" s="15"/>
+      <c r="K37" s="15"/>
+      <c r="L37" s="15">
         <v>3</v>
       </c>
-      <c r="K37" s="14">
+      <c r="M37" s="15">
         <v>0.15</v>
       </c>
-      <c r="L37" s="14"/>
-      <c r="M37" s="14"/>
-      <c r="N37" s="14"/>
-      <c r="O37" s="14"/>
-      <c r="P37" s="14"/>
-      <c r="Q37" s="14"/>
-      <c r="R37" s="14"/>
-      <c r="S37" s="14"/>
-      <c r="T37" s="14">
-        <f t="shared" ref="T37:T40" si="5">D37*E37+F37*G37+H37*I37+J37*K37+L37*M37+N37*O37+P37*Q37+R37*S37</f>
+      <c r="N37" s="15"/>
+      <c r="O37" s="15"/>
+      <c r="P37" s="15"/>
+      <c r="Q37" s="15"/>
+      <c r="R37" s="15"/>
+      <c r="S37" s="15"/>
+      <c r="T37" s="15"/>
+      <c r="U37" s="15"/>
+      <c r="V37" s="15">
+        <f t="shared" si="4"/>
         <v>0.5</v>
       </c>
-      <c r="U37" s="14"/>
-      <c r="W37" s="6"/>
+      <c r="W37" s="15"/>
+      <c r="Y37" s="6"/>
     </row>
-    <row r="38" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A38" s="14"/>
-      <c r="B38" s="14"/>
-      <c r="C38" s="14" t="s">
-        <v>41</v>
-      </c>
-      <c r="D38" s="14">
+    <row r="38" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A38" s="15"/>
+      <c r="B38" s="15"/>
+      <c r="C38" s="15" t="s">
+        <v>43</v>
+      </c>
+      <c r="D38" s="15">
         <v>1</v>
       </c>
-      <c r="E38" s="14">
+      <c r="E38" s="15">
         <v>0.12</v>
       </c>
-      <c r="F38" s="14"/>
-      <c r="G38" s="14"/>
-      <c r="H38" s="14">
+      <c r="F38" s="15"/>
+      <c r="G38" s="15"/>
+      <c r="H38" s="15"/>
+      <c r="I38" s="15"/>
+      <c r="J38" s="15">
         <v>2</v>
       </c>
-      <c r="I38" s="14">
+      <c r="K38" s="15">
         <v>0.08</v>
       </c>
-      <c r="J38" s="14"/>
-      <c r="K38" s="14"/>
-      <c r="L38" s="14"/>
-      <c r="M38" s="14"/>
-      <c r="N38" s="14"/>
-      <c r="O38" s="14"/>
-      <c r="P38" s="14"/>
-      <c r="Q38" s="14"/>
-      <c r="R38" s="14"/>
-      <c r="S38" s="14"/>
-      <c r="T38" s="14">
+      <c r="L38" s="15"/>
+      <c r="M38" s="15"/>
+      <c r="N38" s="15"/>
+      <c r="O38" s="15"/>
+      <c r="P38" s="15"/>
+      <c r="Q38" s="15"/>
+      <c r="R38" s="15"/>
+      <c r="S38" s="15"/>
+      <c r="T38" s="15"/>
+      <c r="U38" s="15"/>
+      <c r="V38" s="15">
+        <f>D38*E38+F38*G38+H38*I38+J38*K38+L38*M38+N38*O38+P38*Q38+R38*S38+T38*U38</f>
+        <v>0.28</v>
+      </c>
+      <c r="W38" s="15"/>
+      <c r="Y38" s="6"/>
+    </row>
+    <row r="39" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
+      <c r="A39" s="20"/>
+      <c r="B39" s="20"/>
+      <c r="C39" s="20"/>
+      <c r="D39" s="20"/>
+      <c r="E39" s="20"/>
+      <c r="F39" s="20"/>
+      <c r="G39" s="20"/>
+      <c r="H39" s="20"/>
+      <c r="I39" s="20"/>
+      <c r="J39" s="20"/>
+      <c r="K39" s="20"/>
+      <c r="L39" s="20"/>
+      <c r="M39" s="20"/>
+      <c r="N39" s="30"/>
+      <c r="O39" s="30"/>
+      <c r="P39" s="30"/>
+      <c r="Q39" s="30"/>
+      <c r="R39" s="30"/>
+      <c r="S39" s="30"/>
+      <c r="T39" s="30"/>
+      <c r="U39" s="30"/>
+      <c r="V39" s="20"/>
+      <c r="W39" s="20"/>
+      <c r="Y39" s="22"/>
+    </row>
+    <row r="40" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
+      <c r="A40" s="15"/>
+      <c r="B40" s="15"/>
+      <c r="C40" s="15" t="s">
+        <v>44</v>
+      </c>
+      <c r="D40" s="15">
+        <v>1</v>
+      </c>
+      <c r="E40" s="15">
+        <v>0.12</v>
+      </c>
+      <c r="F40" s="15">
+        <v>1</v>
+      </c>
+      <c r="G40" s="15">
+        <v>0.05</v>
+      </c>
+      <c r="H40" s="15"/>
+      <c r="I40" s="15"/>
+      <c r="J40" s="15">
+        <v>2</v>
+      </c>
+      <c r="K40" s="15">
+        <v>0.08</v>
+      </c>
+      <c r="L40" s="15">
+        <v>3</v>
+      </c>
+      <c r="M40" s="15">
+        <v>0.08</v>
+      </c>
+      <c r="N40" s="15"/>
+      <c r="O40" s="15"/>
+      <c r="P40" s="15"/>
+      <c r="Q40" s="15"/>
+      <c r="R40" s="15"/>
+      <c r="S40" s="15"/>
+      <c r="T40" s="15"/>
+      <c r="U40" s="15"/>
+      <c r="V40" s="15">
+        <f>D40*E40+F40*G40+H40*I40+J40*K40+L40*M40+N40*O40+P40*Q40+R40*S40+T40*U40</f>
+        <v>0.57</v>
+      </c>
+      <c r="W40" s="15"/>
+      <c r="Y40" s="6"/>
+    </row>
+    <row r="41" s="1" customFormat="1" customHeight="1" spans="1:25">
+      <c r="A41" s="15" t="s">
+        <v>45</v>
+      </c>
+      <c r="B41" s="15"/>
+      <c r="C41" s="15" t="s">
+        <v>46</v>
+      </c>
+      <c r="D41" s="31">
+        <f>SUM(D3:D40)</f>
+        <v>13</v>
+      </c>
+      <c r="E41" s="31">
+        <f>SUM(E3:E40)</f>
+        <v>0.84</v>
+      </c>
+      <c r="F41" s="31">
+        <f>SUM(F3:F40)</f>
+        <v>27</v>
+      </c>
+      <c r="G41" s="31">
+        <f>SUM(G3:G40)</f>
+        <v>0.95</v>
+      </c>
+      <c r="H41" s="31">
+        <f>SUM(H3:H40)</f>
+        <v>0</v>
+      </c>
+      <c r="I41" s="31">
+        <f>SUM(I3:I40)</f>
+        <v>0</v>
+      </c>
+      <c r="J41" s="31">
+        <f t="shared" ref="J41:T41" si="5">SUM(J3:J40)</f>
+        <v>14</v>
+      </c>
+      <c r="K41" s="31">
         <f t="shared" si="5"/>
-        <v>0.28</v>
-      </c>
-      <c r="U38" s="14"/>
-      <c r="W38" s="6"/>
+        <v>0.72</v>
+      </c>
+      <c r="L41" s="31">
+        <f t="shared" si="5"/>
+        <v>17</v>
+      </c>
+      <c r="M41" s="31">
+        <f t="shared" si="5"/>
+        <v>0.55</v>
+      </c>
+      <c r="N41" s="31">
+        <f t="shared" si="5"/>
+        <v>2</v>
+      </c>
+      <c r="O41" s="31">
+        <f t="shared" si="5"/>
+        <v>0.12</v>
+      </c>
+      <c r="P41" s="31">
+        <f t="shared" si="5"/>
+        <v>7</v>
+      </c>
+      <c r="Q41" s="31">
+        <f t="shared" si="5"/>
+        <v>0.6</v>
+      </c>
+      <c r="R41" s="31">
+        <f t="shared" si="5"/>
+        <v>12</v>
+      </c>
+      <c r="S41" s="31">
+        <f t="shared" si="5"/>
+        <v>0.4</v>
+      </c>
+      <c r="T41" s="31">
+        <f>SUM(T3:T40)</f>
+        <v>0</v>
+      </c>
+      <c r="U41" s="31">
+        <f>SUM(U3:U40)</f>
+        <v>0</v>
+      </c>
+      <c r="V41" s="31">
+        <f>SUM(V3:V40)</f>
+        <v>8.34</v>
+      </c>
+      <c r="W41" s="15"/>
+      <c r="Y41" s="6"/>
     </row>
-    <row r="39" s="3" customFormat="1" ht="15" customHeight="1" spans="1:23">
-      <c r="A39" s="18"/>
-      <c r="B39" s="18"/>
-      <c r="C39" s="18"/>
-      <c r="D39" s="18"/>
-      <c r="E39" s="18"/>
-      <c r="F39" s="18"/>
-      <c r="G39" s="18"/>
-      <c r="H39" s="18"/>
-      <c r="I39" s="18"/>
-      <c r="J39" s="18"/>
-      <c r="K39" s="18"/>
-      <c r="L39" s="27"/>
-      <c r="M39" s="27"/>
-      <c r="N39" s="27"/>
-      <c r="O39" s="27"/>
-      <c r="P39" s="27"/>
-      <c r="Q39" s="27"/>
-      <c r="R39" s="35"/>
-      <c r="S39" s="35"/>
-      <c r="T39" s="18"/>
-      <c r="U39" s="18"/>
-      <c r="W39" s="31"/>
+    <row r="42" customHeight="1" spans="1:25">
+      <c r="A42" s="32"/>
+      <c r="B42" s="32"/>
     </row>
-    <row r="40" s="1" customFormat="1" ht="59" customHeight="1" spans="1:23">
-      <c r="A40" s="14"/>
-      <c r="B40" s="14"/>
-      <c r="C40" s="14" t="s">
-        <v>42</v>
-      </c>
-      <c r="D40" s="14">
-        <v>1</v>
-      </c>
-      <c r="E40" s="14">
-        <v>0.12</v>
-      </c>
-      <c r="F40" s="14">
-        <v>1</v>
-      </c>
-      <c r="G40" s="14">
-        <v>0.05</v>
-      </c>
-      <c r="H40" s="14">
-        <v>2</v>
-      </c>
-      <c r="I40" s="14">
-        <v>0.08</v>
-      </c>
-      <c r="J40" s="14">
-        <v>3</v>
-      </c>
-      <c r="K40" s="14">
-        <v>0.08</v>
-      </c>
-      <c r="L40" s="14"/>
-      <c r="M40" s="14"/>
-      <c r="N40" s="14"/>
-      <c r="O40" s="14"/>
-      <c r="P40" s="14"/>
-      <c r="Q40" s="14"/>
-      <c r="R40" s="14"/>
-      <c r="S40" s="14"/>
-      <c r="T40" s="14">
-        <f t="shared" si="5"/>
-        <v>0.57</v>
-      </c>
-      <c r="U40" s="14"/>
-      <c r="W40" s="6"/>
-    </row>
-    <row r="41" s="1" customFormat="1" customHeight="1" spans="1:23">
-      <c r="A41" s="14" t="s">
-        <v>43</v>
-      </c>
-      <c r="B41" s="14"/>
-      <c r="C41" s="14" t="s">
-        <v>44</v>
-      </c>
-      <c r="D41" s="25">
-        <f t="shared" ref="D41:R41" si="6">SUM(D3:D40)</f>
-        <v>13</v>
-      </c>
-      <c r="E41" s="25">
-        <f t="shared" si="6"/>
-        <v>0.84</v>
-      </c>
-      <c r="F41" s="25">
-        <f t="shared" si="6"/>
-        <v>27</v>
-      </c>
-      <c r="G41" s="25">
-        <f t="shared" si="6"/>
-        <v>0.95</v>
-      </c>
-      <c r="H41" s="25">
-        <f t="shared" si="6"/>
-        <v>14</v>
-      </c>
-      <c r="I41" s="25">
-        <f t="shared" si="6"/>
-        <v>0.72</v>
-      </c>
-      <c r="J41" s="25">
-        <f t="shared" si="6"/>
-        <v>17</v>
-      </c>
-      <c r="K41" s="25">
-        <f t="shared" si="6"/>
-        <v>0.55</v>
-      </c>
-      <c r="L41" s="25">
-        <f t="shared" si="6"/>
-        <v>2</v>
-      </c>
-      <c r="M41" s="25">
-        <f t="shared" si="6"/>
-        <v>0.12</v>
-      </c>
-      <c r="N41" s="25">
-        <f t="shared" si="6"/>
-        <v>7</v>
-      </c>
-      <c r="O41" s="25">
-        <f t="shared" si="6"/>
-        <v>0.6</v>
-      </c>
-      <c r="P41" s="25">
-        <f t="shared" si="6"/>
-        <v>12</v>
-      </c>
-      <c r="Q41" s="25">
-        <f t="shared" si="6"/>
-        <v>0.4</v>
-      </c>
-      <c r="R41" s="25"/>
-      <c r="S41" s="25"/>
-      <c r="T41" s="25">
-        <f>SUM(T3:T40)</f>
-        <v>8.34</v>
-      </c>
-      <c r="U41" s="14"/>
-      <c r="W41" s="6"/>
-    </row>
-    <row r="42" customHeight="1" spans="1:2">
-      <c r="A42" s="26"/>
-      <c r="B42" s="26"/>
-    </row>
-    <row r="43" customHeight="1" spans="1:1">
+    <row r="43" customHeight="1" spans="1:25">
       <c r="A43" s="5" t="s">
-        <v>45</v>
+        <v>47</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:U1"/>
+    <mergeCell ref="A1:W1"/>
   </mergeCells>
   <pageMargins left="0.984027777777778" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <pageSetup paperSize="9" scale="40" orientation="portrait"/>
+  <pageSetup paperSize="9" scale="37" orientation="portrait"/>
   <headerFooter/>
   <drawing r:id="rId1"/>
 </worksheet>

</xml_diff>

<commit_message>
feat(internal-quote): map painting material and labor costs separately
</commit_message>
<xml_diff>
--- a/backend/app/data/internal_quote_import_templates/喷油报价单.xlsx
+++ b/backend/app/data/internal_quote_import_templates/喷油报价单.xlsx
@@ -9,7 +9,7 @@
     </mc:Choice>
   </mc:AlternateContent>
   <bookViews>
-    <workbookView windowWidth="24750" windowHeight="12060"/>
+    <workbookView windowWidth="27945" windowHeight="12255"/>
   </bookViews>
   <sheets>
     <sheet name="喷油0923" sheetId="1" r:id="rId1"/>
@@ -716,7 +716,7 @@
     <definedName name="Wire26_8in">#REF!</definedName>
     <definedName name="WORDREPORT">'[4]Home Page'!$AB$1</definedName>
     <definedName name="電子元件表1">#REF!</definedName>
-    <definedName name="_xlnm.Print_Area" localSheetId="0">喷油0923!$A$1:$W$41</definedName>
+    <definedName name="_xlnm.Print_Area" localSheetId="0">喷油0923!$A$1:$Y$41</definedName>
   </definedNames>
   <calcPr calcId="191029"/>
   <extLst>
@@ -736,7 +736,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="53" uniqueCount="48">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="55" uniqueCount="50">
   <si>
     <t>第二代恐龙公园报价</t>
   </si>
@@ -805,6 +805,12 @@
   </si>
   <si>
     <t>总报价</t>
+  </si>
+  <si>
+    <t>油漆</t>
+  </si>
+  <si>
+    <t>人工</t>
   </si>
   <si>
     <t>备注</t>
@@ -1076,7 +1082,7 @@
       <scheme val="minor"/>
     </font>
   </fonts>
-  <fills count="38">
+  <fills count="39">
     <fill>
       <patternFill patternType="none"/>
     </fill>
@@ -1104,6 +1110,12 @@
     <fill>
       <patternFill patternType="solid">
         <fgColor theme="9" tint="0.599993896298105"/>
+        <bgColor indexed="64"/>
+      </patternFill>
+    </fill>
+    <fill>
+      <patternFill patternType="solid">
+        <fgColor rgb="FFFFC000"/>
         <bgColor indexed="64"/>
       </patternFill>
     </fill>
@@ -1473,7 +1485,7 @@
     <xf numFmtId="0" fontId="7" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="0" fillId="9" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="0" fillId="10" borderId="4" applyNumberFormat="0" applyFont="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="8" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
@@ -1497,16 +1509,16 @@
     <xf numFmtId="0" fontId="13" fillId="0" borderId="0" applyNumberFormat="0" applyFill="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="14" fillId="10" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="15" fillId="11" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="16" fillId="11" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="17" fillId="12" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="14" fillId="11" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="15" fillId="12" borderId="8" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="16" fillId="12" borderId="7" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="17" fillId="13" borderId="9" applyNumberFormat="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="18" fillId="0" borderId="10" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
@@ -1515,89 +1527,89 @@
     <xf numFmtId="0" fontId="19" fillId="0" borderId="11" applyNumberFormat="0" applyFill="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="20" fillId="13" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="21" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="22" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="23" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="20" fillId="14" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="21" fillId="15" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="22" fillId="16" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="23" fillId="17" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="18" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="24" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="23" fillId="4" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="19" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="24" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="20" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="21" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="22" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="23" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="24" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="25" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="26" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="27" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="28" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="29" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="30" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="31" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="32" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="33" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="24" fillId="34" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="23" fillId="35" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="24" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="36" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="24" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="24" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="23" fillId="37" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
+    <xf numFmtId="0" fontId="23" fillId="38" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0">
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="33">
+  <cellXfs count="34">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
@@ -1631,6 +1643,9 @@
     <xf numFmtId="0" fontId="2" fillId="5" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -1667,12 +1682,12 @@
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="6" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="2" fillId="7" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
+    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
     <xf numFmtId="0" fontId="2" fillId="3" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
@@ -1691,7 +1706,7 @@
     <xf numFmtId="0" fontId="2" fillId="2" borderId="3" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="8" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+    <xf numFmtId="0" fontId="2" fillId="9" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center"/>
     </xf>
     <xf numFmtId="0" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
@@ -2751,7 +2766,7 @@
   <sheetPr>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:Y43"/>
+  <dimension ref="A1:AA43"/>
   <sheetFormatPr defaultColWidth="11.45" defaultRowHeight="40" customHeight="1"/>
   <cols>
     <col min="1" max="2" width="20.4416666666667" style="5" customWidth="1"/>
@@ -2760,15 +2775,15 @@
     <col min="6" max="6" width="7.5" style="5" customWidth="1"/>
     <col min="7" max="20" width="6.63333333333333" style="5" customWidth="1"/>
     <col min="21" max="21" width="8.89166666666667" style="5" customWidth="1"/>
-    <col min="22" max="22" width="6.63333333333333" style="5" customWidth="1"/>
-    <col min="23" max="23" width="18.2166666666667" style="5" customWidth="1"/>
-    <col min="24" max="24" width="11.45" style="1" customWidth="1"/>
-    <col min="25" max="25" width="11.45" style="6" customWidth="1"/>
-    <col min="26" max="16382" width="11.45" style="1" customWidth="1"/>
+    <col min="22" max="24" width="6.63333333333333" style="5" customWidth="1"/>
+    <col min="25" max="25" width="18.2166666666667" style="5" customWidth="1"/>
+    <col min="26" max="26" width="11.45" style="1" customWidth="1"/>
+    <col min="27" max="27" width="11.45" style="6" customWidth="1"/>
+    <col min="28" max="16382" width="11.45" style="1" customWidth="1"/>
     <col min="16383" max="16384" width="11.45" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" s="1" customFormat="1" customHeight="1" spans="1:25">
+    <row r="1" s="1" customFormat="1" customHeight="1" spans="1:27">
       <c r="A1" s="7" t="s">
         <v>0</v>
       </c>
@@ -2794,9 +2809,11 @@
       <c r="U1" s="7"/>
       <c r="V1" s="7"/>
       <c r="W1" s="7"/>
-      <c r="Y1" s="6"/>
+      <c r="X1" s="7"/>
+      <c r="Y1" s="7"/>
+      <c r="AA1" s="6"/>
     </row>
-    <row r="2" s="2" customFormat="1" customHeight="1" spans="1:25">
+    <row r="2" s="2" customFormat="1" customHeight="1" spans="1:27">
       <c r="A2" s="8" t="s">
         <v>1</v>
       </c>
@@ -2860,1418 +2877,1513 @@
       <c r="U2" s="10" t="s">
         <v>21</v>
       </c>
-      <c r="V2" s="8" t="s">
+      <c r="V2" s="11" t="s">
         <v>22</v>
       </c>
-      <c r="W2" s="8" t="s">
+      <c r="W2" s="9" t="s">
         <v>23</v>
       </c>
-      <c r="Y2" s="11"/>
+      <c r="X2" s="10" t="s">
+        <v>24</v>
+      </c>
+      <c r="Y2" s="8" t="s">
+        <v>25</v>
+      </c>
+      <c r="AA2" s="12"/>
     </row>
-    <row r="3" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A3" s="12"/>
-      <c r="B3" s="12"/>
-      <c r="C3" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D3" s="14"/>
-      <c r="E3" s="15"/>
-      <c r="F3" s="15">
+    <row r="3" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A3" s="13"/>
+      <c r="B3" s="13"/>
+      <c r="C3" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D3" s="15"/>
+      <c r="E3" s="16"/>
+      <c r="F3" s="16">
         <v>2</v>
       </c>
-      <c r="G3" s="15">
+      <c r="G3" s="16">
         <v>0.15</v>
       </c>
-      <c r="H3" s="15"/>
-      <c r="I3" s="15"/>
-      <c r="J3" s="15"/>
-      <c r="K3" s="15"/>
-      <c r="L3" s="15"/>
-      <c r="M3" s="15"/>
-      <c r="N3" s="15"/>
-      <c r="O3" s="15"/>
-      <c r="P3" s="15"/>
-      <c r="Q3" s="15"/>
-      <c r="R3" s="15"/>
-      <c r="S3" s="15"/>
-      <c r="T3" s="15"/>
-      <c r="U3" s="15"/>
-      <c r="V3" s="15">
+      <c r="H3" s="16"/>
+      <c r="I3" s="16"/>
+      <c r="J3" s="16"/>
+      <c r="K3" s="16"/>
+      <c r="L3" s="16"/>
+      <c r="M3" s="16"/>
+      <c r="N3" s="16"/>
+      <c r="O3" s="16"/>
+      <c r="P3" s="16"/>
+      <c r="Q3" s="16"/>
+      <c r="R3" s="16"/>
+      <c r="S3" s="16"/>
+      <c r="T3" s="16"/>
+      <c r="U3" s="16"/>
+      <c r="V3" s="16">
         <f>D3*E3+F3*G3+H3*I3+J3*K3+L3*M3+N3*O3+P3*Q3+R3*S3+T3*U3</f>
         <v>0.3</v>
       </c>
-      <c r="W3" s="15"/>
-      <c r="X3" s="1">
+      <c r="W3" s="16">
+        <v>0.02</v>
+      </c>
+      <c r="X3" s="16">
+        <f>V3-W3</f>
+        <v>0.28</v>
+      </c>
+      <c r="Y3" s="16"/>
+      <c r="Z3" s="1">
         <v>1.77</v>
       </c>
-      <c r="Y3" s="16"/>
+      <c r="AA3" s="17"/>
     </row>
-    <row r="4" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
-      <c r="A4" s="17"/>
-      <c r="B4" s="17"/>
-      <c r="C4" s="18"/>
-      <c r="D4" s="19"/>
-      <c r="E4" s="20"/>
-      <c r="F4" s="20"/>
-      <c r="G4" s="20"/>
-      <c r="H4" s="20"/>
-      <c r="I4" s="20"/>
-      <c r="J4" s="20"/>
-      <c r="K4" s="20"/>
-      <c r="L4" s="20"/>
-      <c r="M4" s="20"/>
-      <c r="N4" s="20"/>
-      <c r="O4" s="20"/>
-      <c r="P4" s="20"/>
-      <c r="Q4" s="20"/>
-      <c r="R4" s="20"/>
-      <c r="S4" s="20"/>
-      <c r="T4" s="20"/>
-      <c r="U4" s="20"/>
-      <c r="V4" s="20"/>
-      <c r="W4" s="20"/>
+    <row r="4" s="3" customFormat="1" ht="15" customHeight="1" spans="1:27">
+      <c r="A4" s="18"/>
+      <c r="B4" s="18"/>
+      <c r="C4" s="19"/>
+      <c r="D4" s="20"/>
+      <c r="E4" s="21"/>
+      <c r="F4" s="21"/>
+      <c r="G4" s="21"/>
+      <c r="H4" s="21"/>
+      <c r="I4" s="21"/>
+      <c r="J4" s="21"/>
+      <c r="K4" s="21"/>
+      <c r="L4" s="21"/>
+      <c r="M4" s="21"/>
+      <c r="N4" s="21"/>
+      <c r="O4" s="21"/>
+      <c r="P4" s="21"/>
+      <c r="Q4" s="21"/>
+      <c r="R4" s="21"/>
+      <c r="S4" s="21"/>
+      <c r="T4" s="21"/>
+      <c r="U4" s="21"/>
+      <c r="V4" s="21"/>
+      <c r="W4" s="21"/>
+      <c r="X4" s="21"/>
       <c r="Y4" s="21"/>
+      <c r="AA4" s="22"/>
     </row>
-    <row r="5" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A5" s="15"/>
-      <c r="B5" s="15"/>
-      <c r="C5" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="D5" s="15"/>
-      <c r="E5" s="15"/>
-      <c r="F5" s="15">
+    <row r="5" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A5" s="16"/>
+      <c r="B5" s="16"/>
+      <c r="C5" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D5" s="16"/>
+      <c r="E5" s="16"/>
+      <c r="F5" s="16">
         <v>2</v>
       </c>
-      <c r="G5" s="15">
+      <c r="G5" s="16">
         <v>0.05</v>
       </c>
-      <c r="H5" s="15"/>
-      <c r="I5" s="15"/>
-      <c r="J5" s="15"/>
-      <c r="K5" s="15"/>
-      <c r="L5" s="15"/>
-      <c r="M5" s="15"/>
-      <c r="N5" s="15"/>
-      <c r="O5" s="15"/>
-      <c r="P5" s="15"/>
-      <c r="Q5" s="15"/>
-      <c r="R5" s="15"/>
-      <c r="S5" s="15"/>
-      <c r="T5" s="15"/>
-      <c r="U5" s="15"/>
-      <c r="V5" s="15">
+      <c r="H5" s="16"/>
+      <c r="I5" s="16"/>
+      <c r="J5" s="16"/>
+      <c r="K5" s="16"/>
+      <c r="L5" s="16"/>
+      <c r="M5" s="16"/>
+      <c r="N5" s="16"/>
+      <c r="O5" s="16"/>
+      <c r="P5" s="16"/>
+      <c r="Q5" s="16"/>
+      <c r="R5" s="16"/>
+      <c r="S5" s="16"/>
+      <c r="T5" s="16"/>
+      <c r="U5" s="16"/>
+      <c r="V5" s="16">
         <f>D5*E5+F5*G5+H5*I5+J5*K5+L5*M5+N5*O5+P5*Q5+R5*S5+T5*U5</f>
         <v>0.1</v>
       </c>
-      <c r="W5" s="15"/>
+      <c r="W5" s="16"/>
+      <c r="X5" s="16"/>
       <c r="Y5" s="16"/>
+      <c r="AA5" s="17"/>
     </row>
-    <row r="6" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A6" s="15"/>
-      <c r="B6" s="15"/>
-      <c r="C6" s="15" t="s">
-        <v>26</v>
-      </c>
-      <c r="D6" s="15"/>
-      <c r="E6" s="15"/>
-      <c r="F6" s="15">
+    <row r="6" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A6" s="16"/>
+      <c r="B6" s="16"/>
+      <c r="C6" s="16" t="s">
+        <v>28</v>
+      </c>
+      <c r="D6" s="16"/>
+      <c r="E6" s="16"/>
+      <c r="F6" s="16">
         <v>4</v>
       </c>
-      <c r="G6" s="15">
+      <c r="G6" s="16">
         <v>0.05</v>
       </c>
-      <c r="H6" s="15"/>
-      <c r="I6" s="15"/>
-      <c r="J6" s="15"/>
-      <c r="K6" s="15"/>
-      <c r="L6" s="15"/>
-      <c r="M6" s="15"/>
-      <c r="N6" s="15"/>
-      <c r="O6" s="15"/>
-      <c r="P6" s="15"/>
-      <c r="Q6" s="15"/>
-      <c r="R6" s="15"/>
-      <c r="S6" s="15"/>
-      <c r="T6" s="15"/>
-      <c r="U6" s="15"/>
-      <c r="V6" s="15">
+      <c r="H6" s="16"/>
+      <c r="I6" s="16"/>
+      <c r="J6" s="16"/>
+      <c r="K6" s="16"/>
+      <c r="L6" s="16"/>
+      <c r="M6" s="16"/>
+      <c r="N6" s="16"/>
+      <c r="O6" s="16"/>
+      <c r="P6" s="16"/>
+      <c r="Q6" s="16"/>
+      <c r="R6" s="16"/>
+      <c r="S6" s="16"/>
+      <c r="T6" s="16"/>
+      <c r="U6" s="16"/>
+      <c r="V6" s="16">
         <f>D6*E6+F6*G6+H6*I6+J6*K6+L6*M6+N6*O6+P6*Q6+R6*S6+T6*U6</f>
         <v>0.2</v>
       </c>
-      <c r="W6" s="15"/>
+      <c r="W6" s="16"/>
+      <c r="X6" s="16"/>
       <c r="Y6" s="16"/>
+      <c r="AA6" s="17"/>
     </row>
-    <row r="7" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A7" s="15"/>
-      <c r="B7" s="15"/>
-      <c r="C7" s="15" t="s">
-        <v>27</v>
-      </c>
-      <c r="D7" s="15"/>
-      <c r="E7" s="15"/>
-      <c r="F7" s="15">
+    <row r="7" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A7" s="16"/>
+      <c r="B7" s="16"/>
+      <c r="C7" s="16" t="s">
+        <v>29</v>
+      </c>
+      <c r="D7" s="16"/>
+      <c r="E7" s="16"/>
+      <c r="F7" s="16">
         <v>2</v>
       </c>
-      <c r="G7" s="15">
+      <c r="G7" s="16">
         <v>0.05</v>
       </c>
-      <c r="H7" s="15"/>
-      <c r="I7" s="15"/>
-      <c r="J7" s="15"/>
-      <c r="K7" s="15"/>
-      <c r="L7" s="15"/>
-      <c r="M7" s="15"/>
-      <c r="N7" s="15"/>
-      <c r="O7" s="15"/>
-      <c r="P7" s="15"/>
-      <c r="Q7" s="15"/>
-      <c r="R7" s="15"/>
-      <c r="S7" s="15"/>
-      <c r="T7" s="15"/>
-      <c r="U7" s="15"/>
-      <c r="V7" s="15">
+      <c r="H7" s="16"/>
+      <c r="I7" s="16"/>
+      <c r="J7" s="16"/>
+      <c r="K7" s="16"/>
+      <c r="L7" s="16"/>
+      <c r="M7" s="16"/>
+      <c r="N7" s="16"/>
+      <c r="O7" s="16"/>
+      <c r="P7" s="16"/>
+      <c r="Q7" s="16"/>
+      <c r="R7" s="16"/>
+      <c r="S7" s="16"/>
+      <c r="T7" s="16"/>
+      <c r="U7" s="16"/>
+      <c r="V7" s="16">
         <f t="shared" ref="V7:V12" si="0">D7*E7+F7*G7+H7*I7+J7*K7+L7*M7+N7*O7+P7*Q7+R7*S7+T7*U7</f>
         <v>0.1</v>
       </c>
-      <c r="W7" s="15"/>
+      <c r="W7" s="16"/>
+      <c r="X7" s="16"/>
       <c r="Y7" s="16"/>
+      <c r="AA7" s="17"/>
     </row>
-    <row r="8" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A8" s="15"/>
-      <c r="B8" s="15"/>
-      <c r="C8" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="D8" s="15"/>
-      <c r="E8" s="15"/>
-      <c r="F8" s="15">
+    <row r="8" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A8" s="16"/>
+      <c r="B8" s="16"/>
+      <c r="C8" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D8" s="16"/>
+      <c r="E8" s="16"/>
+      <c r="F8" s="16">
         <v>2</v>
       </c>
-      <c r="G8" s="15">
+      <c r="G8" s="16">
         <v>0.05</v>
       </c>
-      <c r="H8" s="15"/>
-      <c r="I8" s="15"/>
-      <c r="J8" s="15"/>
-      <c r="K8" s="15"/>
-      <c r="L8" s="15"/>
-      <c r="M8" s="15"/>
-      <c r="N8" s="15"/>
-      <c r="O8" s="15"/>
-      <c r="P8" s="15"/>
-      <c r="Q8" s="15"/>
-      <c r="R8" s="15"/>
-      <c r="S8" s="15"/>
-      <c r="T8" s="15"/>
-      <c r="U8" s="15"/>
-      <c r="V8" s="15">
+      <c r="H8" s="16"/>
+      <c r="I8" s="16"/>
+      <c r="J8" s="16"/>
+      <c r="K8" s="16"/>
+      <c r="L8" s="16"/>
+      <c r="M8" s="16"/>
+      <c r="N8" s="16"/>
+      <c r="O8" s="16"/>
+      <c r="P8" s="16"/>
+      <c r="Q8" s="16"/>
+      <c r="R8" s="16"/>
+      <c r="S8" s="16"/>
+      <c r="T8" s="16"/>
+      <c r="U8" s="16"/>
+      <c r="V8" s="16">
         <f t="shared" si="0"/>
         <v>0.1</v>
       </c>
-      <c r="W8" s="15"/>
-      <c r="Y8" s="6"/>
+      <c r="W8" s="16"/>
+      <c r="X8" s="16"/>
+      <c r="Y8" s="16"/>
+      <c r="AA8" s="6"/>
     </row>
-    <row r="9" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A9" s="15"/>
-      <c r="B9" s="15"/>
-      <c r="C9" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D9" s="15"/>
-      <c r="E9" s="15"/>
-      <c r="F9" s="15">
+    <row r="9" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A9" s="16"/>
+      <c r="B9" s="16"/>
+      <c r="C9" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="D9" s="16"/>
+      <c r="E9" s="16"/>
+      <c r="F9" s="16">
         <v>1</v>
       </c>
-      <c r="G9" s="15">
+      <c r="G9" s="16">
         <v>0.05</v>
       </c>
-      <c r="H9" s="15"/>
-      <c r="I9" s="15"/>
-      <c r="J9" s="15"/>
-      <c r="K9" s="15"/>
-      <c r="L9" s="15"/>
-      <c r="M9" s="15"/>
-      <c r="N9" s="15"/>
-      <c r="O9" s="15"/>
-      <c r="P9" s="15"/>
-      <c r="Q9" s="15"/>
-      <c r="R9" s="15"/>
-      <c r="S9" s="15"/>
-      <c r="T9" s="15"/>
-      <c r="U9" s="15"/>
-      <c r="V9" s="15">
+      <c r="H9" s="16"/>
+      <c r="I9" s="16"/>
+      <c r="J9" s="16"/>
+      <c r="K9" s="16"/>
+      <c r="L9" s="16"/>
+      <c r="M9" s="16"/>
+      <c r="N9" s="16"/>
+      <c r="O9" s="16"/>
+      <c r="P9" s="16"/>
+      <c r="Q9" s="16"/>
+      <c r="R9" s="16"/>
+      <c r="S9" s="16"/>
+      <c r="T9" s="16"/>
+      <c r="U9" s="16"/>
+      <c r="V9" s="16">
         <f t="shared" si="0"/>
         <v>0.05</v>
       </c>
-      <c r="W9" s="15"/>
-      <c r="Y9" s="6"/>
+      <c r="W9" s="16"/>
+      <c r="X9" s="16"/>
+      <c r="Y9" s="16"/>
+      <c r="AA9" s="6"/>
     </row>
-    <row r="10" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A10" s="15"/>
-      <c r="B10" s="15"/>
-      <c r="C10" s="15" t="s">
-        <v>30</v>
-      </c>
-      <c r="D10" s="15"/>
-      <c r="E10" s="15"/>
-      <c r="F10" s="15"/>
-      <c r="G10" s="15"/>
-      <c r="H10" s="15"/>
-      <c r="I10" s="15"/>
-      <c r="J10" s="15">
+    <row r="10" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A10" s="16"/>
+      <c r="B10" s="16"/>
+      <c r="C10" s="16" t="s">
+        <v>32</v>
+      </c>
+      <c r="D10" s="16"/>
+      <c r="E10" s="16"/>
+      <c r="F10" s="16"/>
+      <c r="G10" s="16"/>
+      <c r="H10" s="16"/>
+      <c r="I10" s="16"/>
+      <c r="J10" s="16">
         <v>2</v>
       </c>
-      <c r="K10" s="15">
+      <c r="K10" s="16">
         <v>0.08</v>
       </c>
-      <c r="L10" s="15">
+      <c r="L10" s="16">
         <v>1</v>
       </c>
-      <c r="M10" s="15">
+      <c r="M10" s="16">
         <v>0.08</v>
       </c>
-      <c r="N10" s="15"/>
-      <c r="O10" s="15"/>
-      <c r="P10" s="15"/>
-      <c r="Q10" s="15"/>
-      <c r="R10" s="15"/>
-      <c r="S10" s="15"/>
-      <c r="T10" s="15"/>
-      <c r="U10" s="15"/>
-      <c r="V10" s="15">
+      <c r="N10" s="16"/>
+      <c r="O10" s="16"/>
+      <c r="P10" s="16"/>
+      <c r="Q10" s="16"/>
+      <c r="R10" s="16"/>
+      <c r="S10" s="16"/>
+      <c r="T10" s="16"/>
+      <c r="U10" s="16"/>
+      <c r="V10" s="16">
         <f t="shared" si="0"/>
         <v>0.24</v>
       </c>
-      <c r="W10" s="15"/>
-      <c r="Y10" s="6"/>
+      <c r="W10" s="16"/>
+      <c r="X10" s="16"/>
+      <c r="Y10" s="16"/>
+      <c r="AA10" s="6"/>
     </row>
-    <row r="11" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
-      <c r="A11" s="20"/>
-      <c r="B11" s="20"/>
-      <c r="C11" s="20"/>
-      <c r="D11" s="20"/>
-      <c r="E11" s="20"/>
-      <c r="F11" s="20"/>
-      <c r="G11" s="20"/>
-      <c r="H11" s="20"/>
-      <c r="I11" s="20"/>
-      <c r="J11" s="20"/>
-      <c r="K11" s="20"/>
-      <c r="L11" s="20"/>
-      <c r="M11" s="20"/>
-      <c r="N11" s="20"/>
-      <c r="O11" s="20"/>
-      <c r="P11" s="20"/>
-      <c r="Q11" s="20"/>
-      <c r="R11" s="20"/>
-      <c r="S11" s="20"/>
-      <c r="T11" s="20"/>
-      <c r="U11" s="20"/>
-      <c r="V11" s="20"/>
-      <c r="W11" s="20"/>
-      <c r="Y11" s="22"/>
+    <row r="11" s="3" customFormat="1" ht="15" customHeight="1" spans="1:27">
+      <c r="A11" s="21"/>
+      <c r="B11" s="21"/>
+      <c r="C11" s="21"/>
+      <c r="D11" s="21"/>
+      <c r="E11" s="21"/>
+      <c r="F11" s="21"/>
+      <c r="G11" s="21"/>
+      <c r="H11" s="21"/>
+      <c r="I11" s="21"/>
+      <c r="J11" s="21"/>
+      <c r="K11" s="21"/>
+      <c r="L11" s="21"/>
+      <c r="M11" s="21"/>
+      <c r="N11" s="21"/>
+      <c r="O11" s="21"/>
+      <c r="P11" s="21"/>
+      <c r="Q11" s="21"/>
+      <c r="R11" s="21"/>
+      <c r="S11" s="21"/>
+      <c r="T11" s="21"/>
+      <c r="U11" s="21"/>
+      <c r="V11" s="21"/>
+      <c r="W11" s="21"/>
+      <c r="X11" s="21"/>
+      <c r="Y11" s="21"/>
+      <c r="AA11" s="23"/>
     </row>
-    <row r="12" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A12" s="15"/>
-      <c r="B12" s="15"/>
-      <c r="C12" s="15" t="s">
-        <v>31</v>
-      </c>
-      <c r="D12" s="15"/>
-      <c r="E12" s="15"/>
-      <c r="F12" s="23"/>
-      <c r="G12" s="15"/>
-      <c r="H12" s="15"/>
-      <c r="I12" s="15"/>
-      <c r="J12" s="15"/>
-      <c r="K12" s="15"/>
-      <c r="L12" s="15"/>
-      <c r="M12" s="15"/>
-      <c r="N12" s="15"/>
-      <c r="O12" s="15"/>
-      <c r="P12" s="15">
+    <row r="12" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A12" s="16"/>
+      <c r="B12" s="16"/>
+      <c r="C12" s="16" t="s">
+        <v>33</v>
+      </c>
+      <c r="D12" s="16"/>
+      <c r="E12" s="16"/>
+      <c r="F12" s="24"/>
+      <c r="G12" s="16"/>
+      <c r="H12" s="16"/>
+      <c r="I12" s="16"/>
+      <c r="J12" s="16"/>
+      <c r="K12" s="16"/>
+      <c r="L12" s="16"/>
+      <c r="M12" s="16"/>
+      <c r="N12" s="16"/>
+      <c r="O12" s="16"/>
+      <c r="P12" s="16">
         <v>1</v>
       </c>
-      <c r="Q12" s="15">
+      <c r="Q12" s="16">
         <v>0.1</v>
       </c>
-      <c r="R12" s="15"/>
-      <c r="S12" s="15"/>
-      <c r="T12" s="15"/>
-      <c r="U12" s="15"/>
-      <c r="V12" s="15">
+      <c r="R12" s="16"/>
+      <c r="S12" s="16"/>
+      <c r="T12" s="16"/>
+      <c r="U12" s="16"/>
+      <c r="V12" s="16">
         <f t="shared" si="0"/>
         <v>0.1</v>
       </c>
-      <c r="W12" s="23"/>
-      <c r="Y12" s="6"/>
+      <c r="W12" s="16"/>
+      <c r="X12" s="16"/>
+      <c r="Y12" s="24"/>
+      <c r="AA12" s="6"/>
     </row>
-    <row r="13" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
-      <c r="A13" s="20"/>
-      <c r="B13" s="20"/>
-      <c r="C13" s="20"/>
-      <c r="D13" s="20"/>
-      <c r="E13" s="20"/>
-      <c r="F13" s="20"/>
-      <c r="G13" s="20"/>
-      <c r="H13" s="20"/>
-      <c r="I13" s="20"/>
-      <c r="J13" s="20"/>
-      <c r="K13" s="20"/>
-      <c r="L13" s="20"/>
-      <c r="M13" s="20"/>
-      <c r="N13" s="20"/>
-      <c r="O13" s="20"/>
-      <c r="P13" s="20"/>
-      <c r="Q13" s="20"/>
-      <c r="R13" s="20"/>
-      <c r="S13" s="20"/>
-      <c r="T13" s="20"/>
-      <c r="U13" s="20"/>
-      <c r="V13" s="20"/>
-      <c r="W13" s="20"/>
-      <c r="Y13" s="22"/>
+    <row r="13" s="3" customFormat="1" ht="15" customHeight="1" spans="1:27">
+      <c r="A13" s="21"/>
+      <c r="B13" s="21"/>
+      <c r="C13" s="21"/>
+      <c r="D13" s="21"/>
+      <c r="E13" s="21"/>
+      <c r="F13" s="21"/>
+      <c r="G13" s="21"/>
+      <c r="H13" s="21"/>
+      <c r="I13" s="21"/>
+      <c r="J13" s="21"/>
+      <c r="K13" s="21"/>
+      <c r="L13" s="21"/>
+      <c r="M13" s="21"/>
+      <c r="N13" s="21"/>
+      <c r="O13" s="21"/>
+      <c r="P13" s="21"/>
+      <c r="Q13" s="21"/>
+      <c r="R13" s="21"/>
+      <c r="S13" s="21"/>
+      <c r="T13" s="21"/>
+      <c r="U13" s="21"/>
+      <c r="V13" s="21"/>
+      <c r="W13" s="21"/>
+      <c r="X13" s="21"/>
+      <c r="Y13" s="21"/>
+      <c r="AA13" s="23"/>
     </row>
-    <row r="14" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A14" s="15"/>
-      <c r="B14" s="15"/>
-      <c r="C14" s="15" t="s">
-        <v>32</v>
-      </c>
-      <c r="D14" s="15"/>
-      <c r="E14" s="15"/>
-      <c r="F14" s="15"/>
-      <c r="G14" s="15"/>
-      <c r="H14" s="15"/>
-      <c r="I14" s="15"/>
-      <c r="J14" s="24">
+    <row r="14" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A14" s="16"/>
+      <c r="B14" s="16"/>
+      <c r="C14" s="16" t="s">
+        <v>34</v>
+      </c>
+      <c r="D14" s="16"/>
+      <c r="E14" s="16"/>
+      <c r="F14" s="16"/>
+      <c r="G14" s="16"/>
+      <c r="H14" s="16"/>
+      <c r="I14" s="16"/>
+      <c r="J14" s="25">
         <v>1</v>
       </c>
-      <c r="K14" s="24">
+      <c r="K14" s="25">
         <v>0.08</v>
       </c>
-      <c r="L14" s="15"/>
-      <c r="M14" s="15"/>
-      <c r="N14" s="15"/>
-      <c r="O14" s="15"/>
-      <c r="P14" s="15">
+      <c r="L14" s="16"/>
+      <c r="M14" s="16"/>
+      <c r="N14" s="16"/>
+      <c r="O14" s="16"/>
+      <c r="P14" s="16">
         <v>1</v>
       </c>
-      <c r="Q14" s="15">
+      <c r="Q14" s="16">
         <v>0.1</v>
       </c>
-      <c r="R14" s="15"/>
-      <c r="S14" s="15"/>
-      <c r="T14" s="15"/>
-      <c r="U14" s="15"/>
-      <c r="V14" s="15">
+      <c r="R14" s="16"/>
+      <c r="S14" s="16"/>
+      <c r="T14" s="16"/>
+      <c r="U14" s="16"/>
+      <c r="V14" s="16">
         <f t="shared" ref="V14:V16" si="1">D14*E14+F14*G14+H14*I14+J14*K14+L14*M14+N14*O14+P14*Q14+R14*S14+T14*U14</f>
         <v>0.18</v>
       </c>
-      <c r="W14" s="15"/>
-      <c r="Y14" s="6"/>
+      <c r="W14" s="16"/>
+      <c r="X14" s="16"/>
+      <c r="Y14" s="16"/>
+      <c r="AA14" s="6"/>
     </row>
-    <row r="15" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A15" s="15"/>
-      <c r="B15" s="15"/>
-      <c r="C15" s="15" t="s">
-        <v>33</v>
-      </c>
-      <c r="D15" s="15"/>
-      <c r="E15" s="15"/>
-      <c r="F15" s="15"/>
-      <c r="G15" s="15"/>
-      <c r="H15" s="15"/>
-      <c r="I15" s="15"/>
-      <c r="J15" s="15">
+    <row r="15" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A15" s="16"/>
+      <c r="B15" s="16"/>
+      <c r="C15" s="16" t="s">
+        <v>35</v>
+      </c>
+      <c r="D15" s="16"/>
+      <c r="E15" s="16"/>
+      <c r="F15" s="16"/>
+      <c r="G15" s="16"/>
+      <c r="H15" s="16"/>
+      <c r="I15" s="16"/>
+      <c r="J15" s="16">
         <v>2</v>
       </c>
-      <c r="K15" s="15">
+      <c r="K15" s="16">
         <v>0.08</v>
       </c>
-      <c r="L15" s="15"/>
-      <c r="M15" s="15"/>
-      <c r="N15" s="15"/>
-      <c r="O15" s="15"/>
-      <c r="P15" s="15"/>
-      <c r="Q15" s="15"/>
-      <c r="R15" s="15"/>
-      <c r="S15" s="15"/>
-      <c r="T15" s="15"/>
-      <c r="U15" s="15"/>
-      <c r="V15" s="15">
+      <c r="L15" s="16"/>
+      <c r="M15" s="16"/>
+      <c r="N15" s="16"/>
+      <c r="O15" s="16"/>
+      <c r="P15" s="16"/>
+      <c r="Q15" s="16"/>
+      <c r="R15" s="16"/>
+      <c r="S15" s="16"/>
+      <c r="T15" s="16"/>
+      <c r="U15" s="16"/>
+      <c r="V15" s="16">
         <f t="shared" si="1"/>
         <v>0.16</v>
       </c>
-      <c r="W15" s="15"/>
-      <c r="Y15" s="6"/>
+      <c r="W15" s="16"/>
+      <c r="X15" s="16"/>
+      <c r="Y15" s="16"/>
+      <c r="AA15" s="6"/>
     </row>
-    <row r="16" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A16" s="15"/>
-      <c r="B16" s="15"/>
-      <c r="C16" s="15" t="s">
-        <v>34</v>
-      </c>
-      <c r="D16" s="15"/>
-      <c r="E16" s="15"/>
-      <c r="F16" s="15"/>
-      <c r="G16" s="15"/>
-      <c r="H16" s="15"/>
-      <c r="I16" s="15"/>
-      <c r="J16" s="24">
+    <row r="16" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A16" s="16"/>
+      <c r="B16" s="16"/>
+      <c r="C16" s="16" t="s">
+        <v>36</v>
+      </c>
+      <c r="D16" s="16"/>
+      <c r="E16" s="16"/>
+      <c r="F16" s="16"/>
+      <c r="G16" s="16"/>
+      <c r="H16" s="16"/>
+      <c r="I16" s="16"/>
+      <c r="J16" s="25">
         <v>1</v>
       </c>
-      <c r="K16" s="24">
+      <c r="K16" s="25">
         <v>0.08</v>
       </c>
-      <c r="L16" s="15"/>
-      <c r="M16" s="15"/>
-      <c r="N16" s="15"/>
-      <c r="O16" s="15"/>
-      <c r="P16" s="15"/>
-      <c r="Q16" s="15"/>
-      <c r="R16" s="15"/>
-      <c r="S16" s="15"/>
-      <c r="T16" s="15"/>
-      <c r="U16" s="15"/>
-      <c r="V16" s="15">
+      <c r="L16" s="16"/>
+      <c r="M16" s="16"/>
+      <c r="N16" s="16"/>
+      <c r="O16" s="16"/>
+      <c r="P16" s="16"/>
+      <c r="Q16" s="16"/>
+      <c r="R16" s="16"/>
+      <c r="S16" s="16"/>
+      <c r="T16" s="16"/>
+      <c r="U16" s="16"/>
+      <c r="V16" s="16">
         <f t="shared" si="1"/>
         <v>0.08</v>
       </c>
-      <c r="W16" s="15"/>
-      <c r="Y16" s="6"/>
+      <c r="W16" s="16"/>
+      <c r="X16" s="16"/>
+      <c r="Y16" s="16"/>
+      <c r="AA16" s="6"/>
     </row>
-    <row r="17" s="4" customFormat="1" ht="20" customHeight="1" spans="1:25">
-      <c r="A17" s="25"/>
-      <c r="B17" s="25"/>
-      <c r="C17" s="25"/>
-      <c r="D17" s="25"/>
-      <c r="E17" s="25"/>
-      <c r="F17" s="25"/>
-      <c r="G17" s="25"/>
-      <c r="H17" s="25"/>
-      <c r="I17" s="25"/>
-      <c r="J17" s="25"/>
-      <c r="K17" s="25"/>
-      <c r="L17" s="25"/>
-      <c r="M17" s="25"/>
-      <c r="N17" s="25"/>
-      <c r="O17" s="25"/>
-      <c r="P17" s="25"/>
-      <c r="Q17" s="25"/>
-      <c r="R17" s="25"/>
-      <c r="S17" s="25"/>
-      <c r="T17" s="25"/>
-      <c r="U17" s="25"/>
-      <c r="V17" s="25"/>
-      <c r="W17" s="25"/>
+    <row r="17" s="4" customFormat="1" ht="20" customHeight="1" spans="1:27">
+      <c r="A17" s="26"/>
+      <c r="B17" s="26"/>
+      <c r="C17" s="26"/>
+      <c r="D17" s="26"/>
+      <c r="E17" s="26"/>
+      <c r="F17" s="26"/>
+      <c r="G17" s="26"/>
+      <c r="H17" s="26"/>
+      <c r="I17" s="26"/>
+      <c r="J17" s="26"/>
+      <c r="K17" s="26"/>
+      <c r="L17" s="26"/>
+      <c r="M17" s="26"/>
+      <c r="N17" s="26"/>
+      <c r="O17" s="26"/>
+      <c r="P17" s="26"/>
+      <c r="Q17" s="26"/>
+      <c r="R17" s="26"/>
+      <c r="S17" s="26"/>
+      <c r="T17" s="26"/>
+      <c r="U17" s="26"/>
+      <c r="V17" s="26"/>
+      <c r="W17" s="26"/>
+      <c r="X17" s="26"/>
       <c r="Y17" s="26"/>
+      <c r="AA17" s="27"/>
     </row>
-    <row r="18" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A18" s="15"/>
-      <c r="B18" s="13"/>
-      <c r="C18" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D18" s="14"/>
-      <c r="E18" s="15"/>
-      <c r="F18" s="15">
+    <row r="18" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A18" s="16"/>
+      <c r="B18" s="14"/>
+      <c r="C18" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D18" s="15"/>
+      <c r="E18" s="16"/>
+      <c r="F18" s="16">
         <v>2</v>
       </c>
-      <c r="G18" s="15">
+      <c r="G18" s="16">
         <v>0.15</v>
       </c>
-      <c r="H18" s="15"/>
-      <c r="I18" s="15"/>
-      <c r="J18" s="15"/>
-      <c r="K18" s="15"/>
-      <c r="L18" s="15"/>
-      <c r="M18" s="15"/>
-      <c r="N18" s="15"/>
-      <c r="O18" s="15"/>
-      <c r="P18" s="15"/>
-      <c r="Q18" s="15"/>
-      <c r="R18" s="15"/>
-      <c r="S18" s="15"/>
-      <c r="T18" s="15"/>
-      <c r="U18" s="15"/>
-      <c r="V18" s="15">
+      <c r="H18" s="16"/>
+      <c r="I18" s="16"/>
+      <c r="J18" s="16"/>
+      <c r="K18" s="16"/>
+      <c r="L18" s="16"/>
+      <c r="M18" s="16"/>
+      <c r="N18" s="16"/>
+      <c r="O18" s="16"/>
+      <c r="P18" s="16"/>
+      <c r="Q18" s="16"/>
+      <c r="R18" s="16"/>
+      <c r="S18" s="16"/>
+      <c r="T18" s="16"/>
+      <c r="U18" s="16"/>
+      <c r="V18" s="16">
         <f>D18*E18+F18*G18+H18*I18+J18*K18+L18*M18+N18*O18+P18*Q18+R18*S18+T18*U18</f>
         <v>0.3</v>
       </c>
-      <c r="W18" s="15"/>
-      <c r="Y18" s="6"/>
+      <c r="W18" s="16"/>
+      <c r="X18" s="16"/>
+      <c r="Y18" s="16"/>
+      <c r="AA18" s="6"/>
     </row>
-    <row r="19" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
-      <c r="A19" s="20"/>
-      <c r="B19" s="18"/>
-      <c r="C19" s="18"/>
-      <c r="D19" s="19"/>
-      <c r="E19" s="20"/>
-      <c r="F19" s="20"/>
-      <c r="G19" s="20"/>
-      <c r="H19" s="20"/>
-      <c r="I19" s="20"/>
-      <c r="J19" s="20"/>
-      <c r="K19" s="20"/>
-      <c r="L19" s="20"/>
-      <c r="M19" s="20"/>
-      <c r="N19" s="20"/>
-      <c r="O19" s="20"/>
-      <c r="P19" s="20"/>
-      <c r="Q19" s="20"/>
-      <c r="R19" s="20"/>
-      <c r="S19" s="20"/>
-      <c r="T19" s="20"/>
-      <c r="U19" s="20"/>
-      <c r="V19" s="20"/>
-      <c r="W19" s="20"/>
-      <c r="Y19" s="22"/>
+    <row r="19" s="3" customFormat="1" ht="15" customHeight="1" spans="1:27">
+      <c r="A19" s="21"/>
+      <c r="B19" s="19"/>
+      <c r="C19" s="19"/>
+      <c r="D19" s="20"/>
+      <c r="E19" s="21"/>
+      <c r="F19" s="21"/>
+      <c r="G19" s="21"/>
+      <c r="H19" s="21"/>
+      <c r="I19" s="21"/>
+      <c r="J19" s="21"/>
+      <c r="K19" s="21"/>
+      <c r="L19" s="21"/>
+      <c r="M19" s="21"/>
+      <c r="N19" s="21"/>
+      <c r="O19" s="21"/>
+      <c r="P19" s="21"/>
+      <c r="Q19" s="21"/>
+      <c r="R19" s="21"/>
+      <c r="S19" s="21"/>
+      <c r="T19" s="21"/>
+      <c r="U19" s="21"/>
+      <c r="V19" s="21"/>
+      <c r="W19" s="21"/>
+      <c r="X19" s="21"/>
+      <c r="Y19" s="21"/>
+      <c r="AA19" s="23"/>
     </row>
-    <row r="20" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A20" s="15"/>
-      <c r="B20" s="15"/>
-      <c r="C20" s="15" t="s">
-        <v>29</v>
-      </c>
-      <c r="D20" s="15">
+    <row r="20" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A20" s="16"/>
+      <c r="B20" s="16"/>
+      <c r="C20" s="16" t="s">
+        <v>31</v>
+      </c>
+      <c r="D20" s="16">
         <v>3</v>
       </c>
-      <c r="E20" s="15">
+      <c r="E20" s="16">
         <v>0.12</v>
       </c>
-      <c r="F20" s="15">
+      <c r="F20" s="16">
         <v>2</v>
       </c>
-      <c r="G20" s="15">
+      <c r="G20" s="16">
         <v>0.05</v>
       </c>
-      <c r="H20" s="15"/>
-      <c r="I20" s="15"/>
-      <c r="J20" s="15"/>
-      <c r="K20" s="15"/>
-      <c r="L20" s="15"/>
-      <c r="M20" s="15"/>
-      <c r="N20" s="15"/>
-      <c r="O20" s="15"/>
-      <c r="P20" s="15">
+      <c r="H20" s="16"/>
+      <c r="I20" s="16"/>
+      <c r="J20" s="16"/>
+      <c r="K20" s="16"/>
+      <c r="L20" s="16"/>
+      <c r="M20" s="16"/>
+      <c r="N20" s="16"/>
+      <c r="O20" s="16"/>
+      <c r="P20" s="16">
         <v>1</v>
       </c>
-      <c r="Q20" s="15">
+      <c r="Q20" s="16">
         <v>0.1</v>
       </c>
-      <c r="R20" s="15">
+      <c r="R20" s="16">
         <v>2</v>
       </c>
-      <c r="S20" s="15">
+      <c r="S20" s="16">
         <v>0.1</v>
       </c>
-      <c r="T20" s="15"/>
-      <c r="U20" s="15"/>
-      <c r="V20" s="15">
+      <c r="T20" s="16"/>
+      <c r="U20" s="16"/>
+      <c r="V20" s="16">
         <f t="shared" ref="V20:V24" si="2">D20*E20+F20*G20+H20*I20+J20*K20+L20*M20+N20*O20+P20*Q20+R20*S20+T20*U20</f>
         <v>0.76</v>
       </c>
-      <c r="W20" s="15"/>
-      <c r="Y20" s="6"/>
+      <c r="W20" s="16"/>
+      <c r="X20" s="16"/>
+      <c r="Y20" s="16"/>
+      <c r="AA20" s="6"/>
     </row>
-    <row r="21" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A21" s="15"/>
-      <c r="B21" s="15"/>
-      <c r="C21" s="15" t="s">
-        <v>28</v>
-      </c>
-      <c r="D21" s="15">
+    <row r="21" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A21" s="16"/>
+      <c r="B21" s="16"/>
+      <c r="C21" s="16" t="s">
+        <v>30</v>
+      </c>
+      <c r="D21" s="16">
         <v>2</v>
       </c>
-      <c r="E21" s="15">
+      <c r="E21" s="16">
         <v>0.12</v>
       </c>
-      <c r="F21" s="15"/>
-      <c r="G21" s="15"/>
-      <c r="H21" s="15"/>
-      <c r="I21" s="15"/>
-      <c r="J21" s="15"/>
-      <c r="K21" s="15"/>
-      <c r="L21" s="15">
+      <c r="F21" s="16"/>
+      <c r="G21" s="16"/>
+      <c r="H21" s="16"/>
+      <c r="I21" s="16"/>
+      <c r="J21" s="16"/>
+      <c r="K21" s="16"/>
+      <c r="L21" s="16">
         <v>1</v>
       </c>
-      <c r="M21" s="15">
+      <c r="M21" s="16">
         <v>0.08</v>
       </c>
-      <c r="N21" s="15"/>
-      <c r="O21" s="15"/>
-      <c r="P21" s="15">
+      <c r="N21" s="16"/>
+      <c r="O21" s="16"/>
+      <c r="P21" s="16">
         <v>1</v>
       </c>
-      <c r="Q21" s="15">
+      <c r="Q21" s="16">
         <v>0.1</v>
       </c>
-      <c r="R21" s="15">
+      <c r="R21" s="16">
         <v>3</v>
       </c>
-      <c r="S21" s="15">
+      <c r="S21" s="16">
         <v>0.1</v>
       </c>
-      <c r="T21" s="15"/>
-      <c r="U21" s="15"/>
-      <c r="V21" s="15">
+      <c r="T21" s="16"/>
+      <c r="U21" s="16"/>
+      <c r="V21" s="16">
         <f t="shared" si="2"/>
         <v>0.72</v>
       </c>
-      <c r="W21" s="15"/>
-      <c r="Y21" s="6"/>
+      <c r="W21" s="16"/>
+      <c r="X21" s="16"/>
+      <c r="Y21" s="16"/>
+      <c r="AA21" s="6"/>
     </row>
-    <row r="22" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A22" s="15"/>
-      <c r="B22" s="15"/>
-      <c r="C22" s="15" t="s">
-        <v>35</v>
-      </c>
-      <c r="D22" s="15">
+    <row r="22" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A22" s="16"/>
+      <c r="B22" s="16"/>
+      <c r="C22" s="16" t="s">
+        <v>37</v>
+      </c>
+      <c r="D22" s="16">
         <v>1</v>
       </c>
-      <c r="E22" s="15">
+      <c r="E22" s="16">
         <v>0.12</v>
       </c>
-      <c r="F22" s="15"/>
-      <c r="G22" s="15"/>
-      <c r="H22" s="15"/>
-      <c r="I22" s="15"/>
-      <c r="J22" s="15"/>
-      <c r="K22" s="15"/>
-      <c r="L22" s="15"/>
-      <c r="M22" s="15"/>
-      <c r="N22" s="15"/>
-      <c r="O22" s="15"/>
-      <c r="P22" s="15">
+      <c r="F22" s="16"/>
+      <c r="G22" s="16"/>
+      <c r="H22" s="16"/>
+      <c r="I22" s="16"/>
+      <c r="J22" s="16"/>
+      <c r="K22" s="16"/>
+      <c r="L22" s="16"/>
+      <c r="M22" s="16"/>
+      <c r="N22" s="16"/>
+      <c r="O22" s="16"/>
+      <c r="P22" s="16">
         <v>1</v>
       </c>
-      <c r="Q22" s="15">
+      <c r="Q22" s="16">
         <v>0.1</v>
       </c>
-      <c r="R22" s="15">
+      <c r="R22" s="16">
         <v>2</v>
       </c>
-      <c r="S22" s="15">
+      <c r="S22" s="16">
         <v>0.1</v>
       </c>
-      <c r="T22" s="15"/>
-      <c r="U22" s="15"/>
-      <c r="V22" s="15">
+      <c r="T22" s="16"/>
+      <c r="U22" s="16"/>
+      <c r="V22" s="16">
         <f t="shared" si="2"/>
         <v>0.42</v>
       </c>
-      <c r="W22" s="15"/>
-      <c r="Y22" s="6"/>
+      <c r="W22" s="16"/>
+      <c r="X22" s="16"/>
+      <c r="Y22" s="16"/>
+      <c r="AA22" s="6"/>
     </row>
-    <row r="23" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
-      <c r="A23" s="20"/>
-      <c r="B23" s="20"/>
-      <c r="C23" s="20"/>
-      <c r="D23" s="20"/>
-      <c r="E23" s="20"/>
-      <c r="F23" s="20"/>
-      <c r="G23" s="20"/>
-      <c r="H23" s="20"/>
-      <c r="I23" s="20"/>
-      <c r="J23" s="20"/>
-      <c r="K23" s="20"/>
-      <c r="L23" s="20"/>
-      <c r="M23" s="20"/>
-      <c r="N23" s="20"/>
-      <c r="O23" s="20"/>
-      <c r="P23" s="20"/>
-      <c r="Q23" s="20"/>
-      <c r="R23" s="20"/>
-      <c r="S23" s="20"/>
-      <c r="T23" s="20"/>
-      <c r="U23" s="20"/>
-      <c r="V23" s="20"/>
-      <c r="W23" s="20"/>
-      <c r="Y23" s="22"/>
+    <row r="23" s="3" customFormat="1" ht="15" customHeight="1" spans="1:27">
+      <c r="A23" s="21"/>
+      <c r="B23" s="21"/>
+      <c r="C23" s="21"/>
+      <c r="D23" s="21"/>
+      <c r="E23" s="21"/>
+      <c r="F23" s="21"/>
+      <c r="G23" s="21"/>
+      <c r="H23" s="21"/>
+      <c r="I23" s="21"/>
+      <c r="J23" s="21"/>
+      <c r="K23" s="21"/>
+      <c r="L23" s="21"/>
+      <c r="M23" s="21"/>
+      <c r="N23" s="21"/>
+      <c r="O23" s="21"/>
+      <c r="P23" s="21"/>
+      <c r="Q23" s="21"/>
+      <c r="R23" s="21"/>
+      <c r="S23" s="21"/>
+      <c r="T23" s="21"/>
+      <c r="U23" s="21"/>
+      <c r="V23" s="21"/>
+      <c r="W23" s="21"/>
+      <c r="X23" s="21"/>
+      <c r="Y23" s="21"/>
+      <c r="AA23" s="23"/>
     </row>
-    <row r="24" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A24" s="15"/>
-      <c r="B24" s="15"/>
-      <c r="C24" s="15" t="s">
-        <v>36</v>
-      </c>
-      <c r="D24" s="15">
+    <row r="24" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A24" s="16"/>
+      <c r="B24" s="16"/>
+      <c r="C24" s="16" t="s">
+        <v>38</v>
+      </c>
+      <c r="D24" s="16">
         <v>3</v>
       </c>
-      <c r="E24" s="15">
+      <c r="E24" s="16">
         <v>0.12</v>
       </c>
-      <c r="F24" s="23"/>
-      <c r="G24" s="15"/>
-      <c r="H24" s="15"/>
-      <c r="I24" s="15"/>
-      <c r="J24" s="15"/>
-      <c r="K24" s="15"/>
-      <c r="L24" s="15">
+      <c r="F24" s="24"/>
+      <c r="G24" s="16"/>
+      <c r="H24" s="16"/>
+      <c r="I24" s="16"/>
+      <c r="J24" s="16"/>
+      <c r="K24" s="16"/>
+      <c r="L24" s="16">
         <v>8</v>
       </c>
-      <c r="M24" s="15">
+      <c r="M24" s="16">
         <v>0.08</v>
       </c>
-      <c r="N24" s="15"/>
-      <c r="O24" s="15"/>
-      <c r="P24" s="15"/>
-      <c r="Q24" s="15"/>
-      <c r="R24" s="15"/>
-      <c r="S24" s="15"/>
-      <c r="T24" s="15"/>
-      <c r="U24" s="15"/>
-      <c r="V24" s="15">
+      <c r="N24" s="16"/>
+      <c r="O24" s="16"/>
+      <c r="P24" s="16"/>
+      <c r="Q24" s="16"/>
+      <c r="R24" s="16"/>
+      <c r="S24" s="16"/>
+      <c r="T24" s="16"/>
+      <c r="U24" s="16"/>
+      <c r="V24" s="16">
         <f t="shared" si="2"/>
         <v>1</v>
       </c>
-      <c r="W24" s="15"/>
-      <c r="Y24" s="6"/>
+      <c r="W24" s="16"/>
+      <c r="X24" s="16"/>
+      <c r="Y24" s="16"/>
+      <c r="AA24" s="6"/>
     </row>
-    <row r="25" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
-      <c r="A25" s="20"/>
-      <c r="B25" s="20"/>
-      <c r="C25" s="20"/>
-      <c r="D25" s="20"/>
-      <c r="E25" s="20"/>
-      <c r="F25" s="20"/>
-      <c r="G25" s="20"/>
-      <c r="H25" s="20"/>
-      <c r="I25" s="20"/>
-      <c r="J25" s="20"/>
-      <c r="K25" s="20"/>
-      <c r="L25" s="20"/>
-      <c r="M25" s="20"/>
-      <c r="N25" s="20"/>
-      <c r="O25" s="20"/>
-      <c r="P25" s="20"/>
-      <c r="Q25" s="20"/>
-      <c r="R25" s="20"/>
-      <c r="S25" s="20"/>
-      <c r="T25" s="20"/>
-      <c r="U25" s="20"/>
-      <c r="V25" s="20"/>
-      <c r="W25" s="20"/>
-      <c r="Y25" s="22"/>
+    <row r="25" s="3" customFormat="1" ht="15" customHeight="1" spans="1:27">
+      <c r="A25" s="21"/>
+      <c r="B25" s="21"/>
+      <c r="C25" s="21"/>
+      <c r="D25" s="21"/>
+      <c r="E25" s="21"/>
+      <c r="F25" s="21"/>
+      <c r="G25" s="21"/>
+      <c r="H25" s="21"/>
+      <c r="I25" s="21"/>
+      <c r="J25" s="21"/>
+      <c r="K25" s="21"/>
+      <c r="L25" s="21"/>
+      <c r="M25" s="21"/>
+      <c r="N25" s="21"/>
+      <c r="O25" s="21"/>
+      <c r="P25" s="21"/>
+      <c r="Q25" s="21"/>
+      <c r="R25" s="21"/>
+      <c r="S25" s="21"/>
+      <c r="T25" s="21"/>
+      <c r="U25" s="21"/>
+      <c r="V25" s="21"/>
+      <c r="W25" s="21"/>
+      <c r="X25" s="21"/>
+      <c r="Y25" s="21"/>
+      <c r="AA25" s="23"/>
     </row>
-    <row r="26" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A26" s="15"/>
-      <c r="B26" s="15"/>
-      <c r="C26" s="15" t="s">
-        <v>37</v>
-      </c>
-      <c r="D26" s="15"/>
-      <c r="E26" s="15"/>
-      <c r="F26" s="15"/>
-      <c r="G26" s="15"/>
-      <c r="H26" s="15"/>
-      <c r="I26" s="15"/>
-      <c r="J26" s="24">
+    <row r="26" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A26" s="16"/>
+      <c r="B26" s="16"/>
+      <c r="C26" s="16" t="s">
+        <v>39</v>
+      </c>
+      <c r="D26" s="16"/>
+      <c r="E26" s="16"/>
+      <c r="F26" s="16"/>
+      <c r="G26" s="16"/>
+      <c r="H26" s="16"/>
+      <c r="I26" s="16"/>
+      <c r="J26" s="25">
         <v>1</v>
       </c>
-      <c r="K26" s="24">
+      <c r="K26" s="25">
         <v>0.08</v>
       </c>
-      <c r="L26" s="15"/>
-      <c r="M26" s="15"/>
-      <c r="N26" s="15"/>
-      <c r="O26" s="15"/>
-      <c r="P26" s="15"/>
-      <c r="Q26" s="15"/>
-      <c r="R26" s="15"/>
-      <c r="S26" s="15"/>
-      <c r="T26" s="15"/>
-      <c r="U26" s="15"/>
-      <c r="V26" s="15">
+      <c r="L26" s="16"/>
+      <c r="M26" s="16"/>
+      <c r="N26" s="16"/>
+      <c r="O26" s="16"/>
+      <c r="P26" s="16"/>
+      <c r="Q26" s="16"/>
+      <c r="R26" s="16"/>
+      <c r="S26" s="16"/>
+      <c r="T26" s="16"/>
+      <c r="U26" s="16"/>
+      <c r="V26" s="16">
         <f t="shared" ref="V26:V29" si="3">D26*E26+F26*G26+H26*I26+J26*K26+L26*M26+N26*O26+P26*Q26+R26*S26+T26*U26</f>
         <v>0.08</v>
       </c>
-      <c r="W26" s="15"/>
-      <c r="Y26" s="6"/>
+      <c r="W26" s="16"/>
+      <c r="X26" s="16"/>
+      <c r="Y26" s="16"/>
+      <c r="AA26" s="6"/>
     </row>
-    <row r="27" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A27" s="15"/>
-      <c r="B27" s="15"/>
-      <c r="C27" s="15" t="s">
-        <v>38</v>
-      </c>
-      <c r="D27" s="15"/>
-      <c r="E27" s="15"/>
-      <c r="F27" s="15"/>
-      <c r="G27" s="15"/>
-      <c r="H27" s="15"/>
-      <c r="I27" s="15"/>
-      <c r="J27" s="15">
+    <row r="27" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A27" s="16"/>
+      <c r="B27" s="16"/>
+      <c r="C27" s="16" t="s">
+        <v>40</v>
+      </c>
+      <c r="D27" s="16"/>
+      <c r="E27" s="16"/>
+      <c r="F27" s="16"/>
+      <c r="G27" s="16"/>
+      <c r="H27" s="16"/>
+      <c r="I27" s="16"/>
+      <c r="J27" s="16">
         <v>2</v>
       </c>
-      <c r="K27" s="15">
+      <c r="K27" s="16">
         <v>0.08</v>
       </c>
-      <c r="L27" s="15"/>
-      <c r="M27" s="15"/>
-      <c r="N27" s="15"/>
-      <c r="O27" s="15"/>
-      <c r="P27" s="15"/>
-      <c r="Q27" s="15"/>
-      <c r="R27" s="15"/>
-      <c r="S27" s="15"/>
-      <c r="T27" s="15"/>
-      <c r="U27" s="15"/>
-      <c r="V27" s="15">
+      <c r="L27" s="16"/>
+      <c r="M27" s="16"/>
+      <c r="N27" s="16"/>
+      <c r="O27" s="16"/>
+      <c r="P27" s="16"/>
+      <c r="Q27" s="16"/>
+      <c r="R27" s="16"/>
+      <c r="S27" s="16"/>
+      <c r="T27" s="16"/>
+      <c r="U27" s="16"/>
+      <c r="V27" s="16">
         <f t="shared" si="3"/>
         <v>0.16</v>
       </c>
-      <c r="W27" s="27"/>
-      <c r="Y27" s="6"/>
+      <c r="W27" s="16"/>
+      <c r="X27" s="16"/>
+      <c r="Y27" s="28"/>
+      <c r="AA27" s="6"/>
     </row>
-    <row r="28" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
-      <c r="A28" s="20"/>
-      <c r="B28" s="20"/>
-      <c r="C28" s="20"/>
-      <c r="D28" s="20"/>
-      <c r="E28" s="20"/>
-      <c r="F28" s="20"/>
-      <c r="G28" s="20"/>
-      <c r="H28" s="20"/>
-      <c r="I28" s="20"/>
-      <c r="J28" s="20"/>
-      <c r="K28" s="20"/>
-      <c r="L28" s="20"/>
-      <c r="M28" s="20"/>
-      <c r="N28" s="20"/>
-      <c r="O28" s="20"/>
-      <c r="P28" s="20"/>
-      <c r="Q28" s="20"/>
-      <c r="R28" s="20"/>
-      <c r="S28" s="20"/>
-      <c r="T28" s="20"/>
-      <c r="U28" s="20"/>
-      <c r="V28" s="20"/>
-      <c r="W28" s="28"/>
-      <c r="Y28" s="22"/>
+    <row r="28" s="3" customFormat="1" ht="15" customHeight="1" spans="1:27">
+      <c r="A28" s="21"/>
+      <c r="B28" s="21"/>
+      <c r="C28" s="21"/>
+      <c r="D28" s="21"/>
+      <c r="E28" s="21"/>
+      <c r="F28" s="21"/>
+      <c r="G28" s="21"/>
+      <c r="H28" s="21"/>
+      <c r="I28" s="21"/>
+      <c r="J28" s="21"/>
+      <c r="K28" s="21"/>
+      <c r="L28" s="21"/>
+      <c r="M28" s="21"/>
+      <c r="N28" s="21"/>
+      <c r="O28" s="21"/>
+      <c r="P28" s="21"/>
+      <c r="Q28" s="21"/>
+      <c r="R28" s="21"/>
+      <c r="S28" s="21"/>
+      <c r="T28" s="21"/>
+      <c r="U28" s="21"/>
+      <c r="V28" s="21"/>
+      <c r="W28" s="21"/>
+      <c r="X28" s="21"/>
+      <c r="Y28" s="29"/>
+      <c r="AA28" s="23"/>
     </row>
-    <row r="29" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A29" s="15"/>
-      <c r="B29" s="15"/>
-      <c r="C29" s="15" t="s">
-        <v>39</v>
-      </c>
-      <c r="D29" s="15">
+    <row r="29" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A29" s="16"/>
+      <c r="B29" s="16"/>
+      <c r="C29" s="16" t="s">
+        <v>41</v>
+      </c>
+      <c r="D29" s="16">
         <v>2</v>
       </c>
-      <c r="E29" s="15">
+      <c r="E29" s="16">
         <v>0.12</v>
       </c>
-      <c r="F29" s="15"/>
-      <c r="G29" s="15"/>
-      <c r="H29" s="15"/>
-      <c r="I29" s="15"/>
-      <c r="J29" s="24">
+      <c r="F29" s="16"/>
+      <c r="G29" s="16"/>
+      <c r="H29" s="16"/>
+      <c r="I29" s="16"/>
+      <c r="J29" s="25">
         <v>1</v>
       </c>
-      <c r="K29" s="24">
+      <c r="K29" s="25">
         <v>0.08</v>
       </c>
-      <c r="L29" s="15"/>
-      <c r="M29" s="15"/>
-      <c r="N29" s="15"/>
-      <c r="O29" s="15"/>
-      <c r="P29" s="15"/>
-      <c r="Q29" s="15"/>
-      <c r="R29" s="23"/>
-      <c r="S29" s="15"/>
-      <c r="T29" s="15"/>
-      <c r="U29" s="15"/>
-      <c r="V29" s="15">
+      <c r="L29" s="16"/>
+      <c r="M29" s="16"/>
+      <c r="N29" s="16"/>
+      <c r="O29" s="16"/>
+      <c r="P29" s="16"/>
+      <c r="Q29" s="16"/>
+      <c r="R29" s="24"/>
+      <c r="S29" s="16"/>
+      <c r="T29" s="16"/>
+      <c r="U29" s="16"/>
+      <c r="V29" s="16">
         <f t="shared" si="3"/>
         <v>0.32</v>
       </c>
-      <c r="W29" s="15"/>
-      <c r="Y29" s="6"/>
+      <c r="W29" s="16"/>
+      <c r="X29" s="16"/>
+      <c r="Y29" s="16"/>
+      <c r="AA29" s="6"/>
     </row>
-    <row r="30" s="4" customFormat="1" ht="20" customHeight="1" spans="1:25">
-      <c r="A30" s="25"/>
-      <c r="B30" s="25"/>
-      <c r="C30" s="25"/>
-      <c r="D30" s="25"/>
-      <c r="E30" s="25"/>
-      <c r="F30" s="25"/>
-      <c r="G30" s="25"/>
-      <c r="H30" s="25"/>
-      <c r="I30" s="25"/>
-      <c r="J30" s="25"/>
-      <c r="K30" s="25"/>
-      <c r="L30" s="25"/>
-      <c r="M30" s="25"/>
-      <c r="N30" s="25"/>
-      <c r="O30" s="25"/>
-      <c r="P30" s="25"/>
-      <c r="Q30" s="25"/>
-      <c r="R30" s="25"/>
-      <c r="S30" s="25"/>
-      <c r="T30" s="25"/>
-      <c r="U30" s="25"/>
-      <c r="V30" s="25"/>
-      <c r="W30" s="25"/>
+    <row r="30" s="4" customFormat="1" ht="20" customHeight="1" spans="1:27">
+      <c r="A30" s="26"/>
+      <c r="B30" s="26"/>
+      <c r="C30" s="26"/>
+      <c r="D30" s="26"/>
+      <c r="E30" s="26"/>
+      <c r="F30" s="26"/>
+      <c r="G30" s="26"/>
+      <c r="H30" s="26"/>
+      <c r="I30" s="26"/>
+      <c r="J30" s="26"/>
+      <c r="K30" s="26"/>
+      <c r="L30" s="26"/>
+      <c r="M30" s="26"/>
+      <c r="N30" s="26"/>
+      <c r="O30" s="26"/>
+      <c r="P30" s="26"/>
+      <c r="Q30" s="26"/>
+      <c r="R30" s="26"/>
+      <c r="S30" s="26"/>
+      <c r="T30" s="26"/>
+      <c r="U30" s="26"/>
+      <c r="V30" s="26"/>
+      <c r="W30" s="26"/>
+      <c r="X30" s="26"/>
       <c r="Y30" s="26"/>
+      <c r="AA30" s="27"/>
     </row>
-    <row r="31" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A31" s="15"/>
-      <c r="B31" s="13"/>
-      <c r="C31" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="D31" s="29"/>
-      <c r="E31" s="15"/>
-      <c r="F31" s="15">
+    <row r="31" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A31" s="16"/>
+      <c r="B31" s="14"/>
+      <c r="C31" s="14" t="s">
+        <v>26</v>
+      </c>
+      <c r="D31" s="30"/>
+      <c r="E31" s="16"/>
+      <c r="F31" s="16">
         <v>2</v>
       </c>
-      <c r="G31" s="15">
+      <c r="G31" s="16">
         <v>0.15</v>
       </c>
-      <c r="H31" s="15"/>
-      <c r="I31" s="15"/>
-      <c r="J31" s="15"/>
-      <c r="K31" s="15"/>
-      <c r="L31" s="15"/>
-      <c r="M31" s="15"/>
-      <c r="N31" s="15"/>
-      <c r="O31" s="15"/>
-      <c r="P31" s="15"/>
-      <c r="Q31" s="15"/>
-      <c r="R31" s="15"/>
-      <c r="S31" s="15"/>
-      <c r="T31" s="15"/>
-      <c r="U31" s="15"/>
-      <c r="V31" s="15">
+      <c r="H31" s="16"/>
+      <c r="I31" s="16"/>
+      <c r="J31" s="16"/>
+      <c r="K31" s="16"/>
+      <c r="L31" s="16"/>
+      <c r="M31" s="16"/>
+      <c r="N31" s="16"/>
+      <c r="O31" s="16"/>
+      <c r="P31" s="16"/>
+      <c r="Q31" s="16"/>
+      <c r="R31" s="16"/>
+      <c r="S31" s="16"/>
+      <c r="T31" s="16"/>
+      <c r="U31" s="16"/>
+      <c r="V31" s="16">
         <f>D31*E31+F31*G31+H31*I31+J31*K31+L31*M31+N31*O31+P31*Q31+R31*S31+T31*U31</f>
         <v>0.3</v>
       </c>
-      <c r="W31" s="15"/>
-      <c r="Y31" s="6"/>
+      <c r="W31" s="16"/>
+      <c r="X31" s="16"/>
+      <c r="Y31" s="16"/>
+      <c r="AA31" s="6"/>
     </row>
-    <row r="32" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
-      <c r="A32" s="20"/>
-      <c r="B32" s="18"/>
-      <c r="C32" s="18"/>
-      <c r="D32" s="19"/>
-      <c r="E32" s="20"/>
-      <c r="F32" s="20"/>
-      <c r="G32" s="20"/>
-      <c r="H32" s="20"/>
-      <c r="I32" s="20"/>
-      <c r="J32" s="20"/>
-      <c r="K32" s="20"/>
-      <c r="L32" s="20"/>
-      <c r="M32" s="20"/>
-      <c r="N32" s="20"/>
-      <c r="O32" s="20"/>
-      <c r="P32" s="20"/>
-      <c r="Q32" s="20"/>
-      <c r="R32" s="20"/>
-      <c r="S32" s="20"/>
-      <c r="T32" s="20"/>
-      <c r="U32" s="20"/>
-      <c r="V32" s="20"/>
-      <c r="W32" s="20"/>
-      <c r="Y32" s="22"/>
+    <row r="32" s="3" customFormat="1" ht="15" customHeight="1" spans="1:27">
+      <c r="A32" s="21"/>
+      <c r="B32" s="19"/>
+      <c r="C32" s="19"/>
+      <c r="D32" s="20"/>
+      <c r="E32" s="21"/>
+      <c r="F32" s="21"/>
+      <c r="G32" s="21"/>
+      <c r="H32" s="21"/>
+      <c r="I32" s="21"/>
+      <c r="J32" s="21"/>
+      <c r="K32" s="21"/>
+      <c r="L32" s="21"/>
+      <c r="M32" s="21"/>
+      <c r="N32" s="21"/>
+      <c r="O32" s="21"/>
+      <c r="P32" s="21"/>
+      <c r="Q32" s="21"/>
+      <c r="R32" s="21"/>
+      <c r="S32" s="21"/>
+      <c r="T32" s="21"/>
+      <c r="U32" s="21"/>
+      <c r="V32" s="21"/>
+      <c r="W32" s="21"/>
+      <c r="X32" s="21"/>
+      <c r="Y32" s="21"/>
+      <c r="AA32" s="23"/>
     </row>
-    <row r="33" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A33" s="15"/>
-      <c r="B33" s="15"/>
-      <c r="C33" s="15" t="s">
-        <v>40</v>
-      </c>
-      <c r="D33" s="14"/>
-      <c r="E33" s="15"/>
-      <c r="F33" s="15"/>
-      <c r="G33" s="15"/>
-      <c r="H33" s="15"/>
-      <c r="I33" s="15"/>
-      <c r="J33" s="15"/>
-      <c r="K33" s="15"/>
-      <c r="L33" s="15">
+    <row r="33" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A33" s="16"/>
+      <c r="B33" s="16"/>
+      <c r="C33" s="16" t="s">
+        <v>42</v>
+      </c>
+      <c r="D33" s="15"/>
+      <c r="E33" s="16"/>
+      <c r="F33" s="16"/>
+      <c r="G33" s="16"/>
+      <c r="H33" s="16"/>
+      <c r="I33" s="16"/>
+      <c r="J33" s="16"/>
+      <c r="K33" s="16"/>
+      <c r="L33" s="16">
         <v>1</v>
       </c>
-      <c r="M33" s="15">
+      <c r="M33" s="16">
         <v>0.08</v>
       </c>
-      <c r="N33" s="15">
+      <c r="N33" s="16">
         <v>2</v>
       </c>
-      <c r="O33" s="15">
+      <c r="O33" s="16">
         <v>0.12</v>
       </c>
-      <c r="P33" s="15">
+      <c r="P33" s="16">
         <v>2</v>
       </c>
-      <c r="Q33" s="15">
+      <c r="Q33" s="16">
         <v>0.1</v>
       </c>
-      <c r="R33" s="15">
+      <c r="R33" s="16">
         <v>5</v>
       </c>
-      <c r="S33" s="15">
+      <c r="S33" s="16">
         <v>0.1</v>
       </c>
-      <c r="T33" s="15"/>
-      <c r="U33" s="15"/>
-      <c r="V33" s="15">
-        <f t="shared" ref="V33:V37" si="4">D33*E33+F33*G33+H33*I33+J33*K33+L33*M33+N33*O33+P33*Q33+R33*S33+T33*U33</f>
+      <c r="T33" s="16"/>
+      <c r="U33" s="16"/>
+      <c r="V33" s="16">
+        <f t="shared" ref="V33:V38" si="4">D33*E33+F33*G33+H33*I33+J33*K33+L33*M33+N33*O33+P33*Q33+R33*S33+T33*U33</f>
         <v>1.02</v>
       </c>
-      <c r="W33" s="15"/>
-      <c r="Y33" s="6"/>
+      <c r="W33" s="16"/>
+      <c r="X33" s="16"/>
+      <c r="Y33" s="16"/>
+      <c r="AA33" s="6"/>
     </row>
-    <row r="34" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A34" s="15"/>
-      <c r="B34" s="15"/>
-      <c r="C34" s="15" t="s">
-        <v>25</v>
-      </c>
-      <c r="D34" s="15"/>
-      <c r="E34" s="15"/>
-      <c r="F34" s="15">
+    <row r="34" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A34" s="16"/>
+      <c r="B34" s="16"/>
+      <c r="C34" s="16" t="s">
+        <v>27</v>
+      </c>
+      <c r="D34" s="16"/>
+      <c r="E34" s="16"/>
+      <c r="F34" s="16">
         <v>2</v>
       </c>
-      <c r="G34" s="15">
+      <c r="G34" s="16">
         <v>0.05</v>
       </c>
-      <c r="H34" s="15"/>
-      <c r="I34" s="15"/>
-      <c r="J34" s="15"/>
-      <c r="K34" s="15"/>
-      <c r="L34" s="15"/>
-      <c r="M34" s="15"/>
-      <c r="N34" s="15"/>
-      <c r="O34" s="15"/>
-      <c r="P34" s="15"/>
-      <c r="Q34" s="15"/>
-      <c r="R34" s="15"/>
-      <c r="S34" s="15"/>
-      <c r="T34" s="15"/>
-      <c r="U34" s="15"/>
-      <c r="V34" s="15">
+      <c r="H34" s="16"/>
+      <c r="I34" s="16"/>
+      <c r="J34" s="16"/>
+      <c r="K34" s="16"/>
+      <c r="L34" s="16"/>
+      <c r="M34" s="16"/>
+      <c r="N34" s="16"/>
+      <c r="O34" s="16"/>
+      <c r="P34" s="16"/>
+      <c r="Q34" s="16"/>
+      <c r="R34" s="16"/>
+      <c r="S34" s="16"/>
+      <c r="T34" s="16"/>
+      <c r="U34" s="16"/>
+      <c r="V34" s="16">
         <f t="shared" si="4"/>
         <v>0.1</v>
       </c>
-      <c r="W34" s="15"/>
-      <c r="Y34" s="6"/>
+      <c r="W34" s="16"/>
+      <c r="X34" s="16"/>
+      <c r="Y34" s="16"/>
+      <c r="AA34" s="6"/>
     </row>
-    <row r="35" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A35" s="15"/>
-      <c r="B35" s="15"/>
-      <c r="C35" s="15" t="s">
-        <v>41</v>
-      </c>
-      <c r="D35" s="15"/>
-      <c r="E35" s="15"/>
-      <c r="F35" s="15">
+    <row r="35" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A35" s="16"/>
+      <c r="B35" s="16"/>
+      <c r="C35" s="16" t="s">
+        <v>43</v>
+      </c>
+      <c r="D35" s="16"/>
+      <c r="E35" s="16"/>
+      <c r="F35" s="16">
         <v>4</v>
       </c>
-      <c r="G35" s="15">
+      <c r="G35" s="16">
         <v>0.05</v>
       </c>
-      <c r="H35" s="15"/>
-      <c r="I35" s="15"/>
-      <c r="J35" s="15"/>
-      <c r="K35" s="15"/>
-      <c r="L35" s="15"/>
-      <c r="M35" s="15"/>
-      <c r="N35" s="15"/>
-      <c r="O35" s="15"/>
-      <c r="P35" s="15"/>
-      <c r="Q35" s="15"/>
-      <c r="R35" s="15"/>
-      <c r="S35" s="15"/>
-      <c r="T35" s="15"/>
-      <c r="U35" s="15"/>
-      <c r="V35" s="15">
+      <c r="H35" s="16"/>
+      <c r="I35" s="16"/>
+      <c r="J35" s="16"/>
+      <c r="K35" s="16"/>
+      <c r="L35" s="16"/>
+      <c r="M35" s="16"/>
+      <c r="N35" s="16"/>
+      <c r="O35" s="16"/>
+      <c r="P35" s="16"/>
+      <c r="Q35" s="16"/>
+      <c r="R35" s="16"/>
+      <c r="S35" s="16"/>
+      <c r="T35" s="16"/>
+      <c r="U35" s="16"/>
+      <c r="V35" s="16">
         <f t="shared" si="4"/>
         <v>0.2</v>
       </c>
-      <c r="W35" s="15"/>
-      <c r="Y35" s="6"/>
+      <c r="W35" s="16"/>
+      <c r="X35" s="16"/>
+      <c r="Y35" s="16"/>
+      <c r="AA35" s="6"/>
     </row>
-    <row r="36" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
-      <c r="A36" s="20"/>
-      <c r="B36" s="20"/>
-      <c r="C36" s="20"/>
-      <c r="D36" s="20"/>
-      <c r="E36" s="20"/>
-      <c r="F36" s="20"/>
-      <c r="G36" s="20"/>
-      <c r="H36" s="20"/>
-      <c r="I36" s="20"/>
-      <c r="J36" s="20"/>
-      <c r="K36" s="20"/>
-      <c r="L36" s="20"/>
-      <c r="M36" s="20"/>
-      <c r="N36" s="20"/>
-      <c r="O36" s="20"/>
-      <c r="P36" s="20"/>
-      <c r="Q36" s="20"/>
-      <c r="R36" s="20"/>
-      <c r="S36" s="20"/>
-      <c r="T36" s="20"/>
-      <c r="U36" s="20"/>
-      <c r="V36" s="20"/>
-      <c r="W36" s="20"/>
-      <c r="Y36" s="22"/>
+    <row r="36" s="3" customFormat="1" ht="15" customHeight="1" spans="1:27">
+      <c r="A36" s="21"/>
+      <c r="B36" s="21"/>
+      <c r="C36" s="21"/>
+      <c r="D36" s="21"/>
+      <c r="E36" s="21"/>
+      <c r="F36" s="21"/>
+      <c r="G36" s="21"/>
+      <c r="H36" s="21"/>
+      <c r="I36" s="21"/>
+      <c r="J36" s="21"/>
+      <c r="K36" s="21"/>
+      <c r="L36" s="21"/>
+      <c r="M36" s="21"/>
+      <c r="N36" s="21"/>
+      <c r="O36" s="21"/>
+      <c r="P36" s="21"/>
+      <c r="Q36" s="21"/>
+      <c r="R36" s="21"/>
+      <c r="S36" s="21"/>
+      <c r="T36" s="21"/>
+      <c r="U36" s="21"/>
+      <c r="V36" s="21"/>
+      <c r="W36" s="21"/>
+      <c r="X36" s="21"/>
+      <c r="Y36" s="21"/>
+      <c r="AA36" s="23"/>
     </row>
-    <row r="37" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A37" s="15"/>
-      <c r="B37" s="15"/>
-      <c r="C37" s="15" t="s">
-        <v>42</v>
-      </c>
-      <c r="D37" s="15"/>
-      <c r="E37" s="15"/>
-      <c r="F37" s="15">
+    <row r="37" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A37" s="16"/>
+      <c r="B37" s="16"/>
+      <c r="C37" s="16" t="s">
+        <v>44</v>
+      </c>
+      <c r="D37" s="16"/>
+      <c r="E37" s="16"/>
+      <c r="F37" s="16">
         <v>1</v>
       </c>
-      <c r="G37" s="15">
+      <c r="G37" s="16">
         <v>0.05</v>
       </c>
-      <c r="H37" s="15"/>
-      <c r="I37" s="15"/>
-      <c r="J37" s="15"/>
-      <c r="K37" s="15"/>
-      <c r="L37" s="15">
+      <c r="H37" s="16"/>
+      <c r="I37" s="16"/>
+      <c r="J37" s="16"/>
+      <c r="K37" s="16"/>
+      <c r="L37" s="16">
         <v>3</v>
       </c>
-      <c r="M37" s="15">
+      <c r="M37" s="16">
         <v>0.15</v>
       </c>
-      <c r="N37" s="15"/>
-      <c r="O37" s="15"/>
-      <c r="P37" s="15"/>
-      <c r="Q37" s="15"/>
-      <c r="R37" s="15"/>
-      <c r="S37" s="15"/>
-      <c r="T37" s="15"/>
-      <c r="U37" s="15"/>
-      <c r="V37" s="15">
+      <c r="N37" s="16"/>
+      <c r="O37" s="16"/>
+      <c r="P37" s="16"/>
+      <c r="Q37" s="16"/>
+      <c r="R37" s="16"/>
+      <c r="S37" s="16"/>
+      <c r="T37" s="16"/>
+      <c r="U37" s="16"/>
+      <c r="V37" s="16">
         <f t="shared" si="4"/>
         <v>0.5</v>
       </c>
-      <c r="W37" s="15"/>
-      <c r="Y37" s="6"/>
+      <c r="W37" s="16"/>
+      <c r="X37" s="16"/>
+      <c r="Y37" s="16"/>
+      <c r="AA37" s="6"/>
     </row>
-    <row r="38" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A38" s="15"/>
-      <c r="B38" s="15"/>
-      <c r="C38" s="15" t="s">
-        <v>43</v>
-      </c>
-      <c r="D38" s="15">
+    <row r="38" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A38" s="16"/>
+      <c r="B38" s="16"/>
+      <c r="C38" s="16" t="s">
+        <v>45</v>
+      </c>
+      <c r="D38" s="16">
         <v>1</v>
       </c>
-      <c r="E38" s="15">
+      <c r="E38" s="16">
         <v>0.12</v>
       </c>
-      <c r="F38" s="15"/>
-      <c r="G38" s="15"/>
-      <c r="H38" s="15"/>
-      <c r="I38" s="15"/>
-      <c r="J38" s="15">
+      <c r="F38" s="16"/>
+      <c r="G38" s="16"/>
+      <c r="H38" s="16"/>
+      <c r="I38" s="16"/>
+      <c r="J38" s="16">
         <v>2</v>
       </c>
-      <c r="K38" s="15">
+      <c r="K38" s="16">
         <v>0.08</v>
       </c>
-      <c r="L38" s="15"/>
-      <c r="M38" s="15"/>
-      <c r="N38" s="15"/>
-      <c r="O38" s="15"/>
-      <c r="P38" s="15"/>
-      <c r="Q38" s="15"/>
-      <c r="R38" s="15"/>
-      <c r="S38" s="15"/>
-      <c r="T38" s="15"/>
-      <c r="U38" s="15"/>
-      <c r="V38" s="15">
-        <f>D38*E38+F38*G38+H38*I38+J38*K38+L38*M38+N38*O38+P38*Q38+R38*S38+T38*U38</f>
+      <c r="L38" s="16"/>
+      <c r="M38" s="16"/>
+      <c r="N38" s="16"/>
+      <c r="O38" s="16"/>
+      <c r="P38" s="16"/>
+      <c r="Q38" s="16"/>
+      <c r="R38" s="16"/>
+      <c r="S38" s="16"/>
+      <c r="T38" s="16"/>
+      <c r="U38" s="16"/>
+      <c r="V38" s="16">
+        <f t="shared" si="4"/>
         <v>0.28</v>
       </c>
-      <c r="W38" s="15"/>
-      <c r="Y38" s="6"/>
+      <c r="W38" s="16"/>
+      <c r="X38" s="16"/>
+      <c r="Y38" s="16"/>
+      <c r="AA38" s="6"/>
     </row>
-    <row r="39" s="3" customFormat="1" ht="15" customHeight="1" spans="1:25">
-      <c r="A39" s="20"/>
-      <c r="B39" s="20"/>
-      <c r="C39" s="20"/>
-      <c r="D39" s="20"/>
-      <c r="E39" s="20"/>
-      <c r="F39" s="20"/>
-      <c r="G39" s="20"/>
-      <c r="H39" s="20"/>
-      <c r="I39" s="20"/>
-      <c r="J39" s="20"/>
-      <c r="K39" s="20"/>
-      <c r="L39" s="20"/>
-      <c r="M39" s="20"/>
-      <c r="N39" s="30"/>
-      <c r="O39" s="30"/>
-      <c r="P39" s="30"/>
-      <c r="Q39" s="30"/>
-      <c r="R39" s="30"/>
-      <c r="S39" s="30"/>
-      <c r="T39" s="30"/>
-      <c r="U39" s="30"/>
-      <c r="V39" s="20"/>
-      <c r="W39" s="20"/>
-      <c r="Y39" s="22"/>
+    <row r="39" s="3" customFormat="1" ht="15" customHeight="1" spans="1:27">
+      <c r="A39" s="21"/>
+      <c r="B39" s="21"/>
+      <c r="C39" s="21"/>
+      <c r="D39" s="21"/>
+      <c r="E39" s="21"/>
+      <c r="F39" s="21"/>
+      <c r="G39" s="21"/>
+      <c r="H39" s="21"/>
+      <c r="I39" s="21"/>
+      <c r="J39" s="21"/>
+      <c r="K39" s="21"/>
+      <c r="L39" s="21"/>
+      <c r="M39" s="21"/>
+      <c r="N39" s="31"/>
+      <c r="O39" s="31"/>
+      <c r="P39" s="31"/>
+      <c r="Q39" s="31"/>
+      <c r="R39" s="31"/>
+      <c r="S39" s="31"/>
+      <c r="T39" s="31"/>
+      <c r="U39" s="31"/>
+      <c r="V39" s="21"/>
+      <c r="W39" s="21"/>
+      <c r="X39" s="21"/>
+      <c r="Y39" s="21"/>
+      <c r="AA39" s="23"/>
     </row>
-    <row r="40" s="1" customFormat="1" ht="59" customHeight="1" spans="1:25">
-      <c r="A40" s="15"/>
-      <c r="B40" s="15"/>
-      <c r="C40" s="15" t="s">
-        <v>44</v>
-      </c>
-      <c r="D40" s="15">
+    <row r="40" s="1" customFormat="1" ht="59" customHeight="1" spans="1:27">
+      <c r="A40" s="16"/>
+      <c r="B40" s="16"/>
+      <c r="C40" s="16" t="s">
+        <v>46</v>
+      </c>
+      <c r="D40" s="16">
         <v>1</v>
       </c>
-      <c r="E40" s="15">
+      <c r="E40" s="16">
         <v>0.12</v>
       </c>
-      <c r="F40" s="15">
+      <c r="F40" s="16">
         <v>1</v>
       </c>
-      <c r="G40" s="15">
+      <c r="G40" s="16">
         <v>0.05</v>
       </c>
-      <c r="H40" s="15"/>
-      <c r="I40" s="15"/>
-      <c r="J40" s="15">
+      <c r="H40" s="16"/>
+      <c r="I40" s="16"/>
+      <c r="J40" s="16">
         <v>2</v>
       </c>
-      <c r="K40" s="15">
+      <c r="K40" s="16">
         <v>0.08</v>
       </c>
-      <c r="L40" s="15">
+      <c r="L40" s="16">
         <v>3</v>
       </c>
-      <c r="M40" s="15">
+      <c r="M40" s="16">
         <v>0.08</v>
       </c>
-      <c r="N40" s="15"/>
-      <c r="O40" s="15"/>
-      <c r="P40" s="15"/>
-      <c r="Q40" s="15"/>
-      <c r="R40" s="15"/>
-      <c r="S40" s="15"/>
-      <c r="T40" s="15"/>
-      <c r="U40" s="15"/>
-      <c r="V40" s="15">
+      <c r="N40" s="16"/>
+      <c r="O40" s="16"/>
+      <c r="P40" s="16"/>
+      <c r="Q40" s="16"/>
+      <c r="R40" s="16"/>
+      <c r="S40" s="16"/>
+      <c r="T40" s="16"/>
+      <c r="U40" s="16"/>
+      <c r="V40" s="16">
         <f>D40*E40+F40*G40+H40*I40+J40*K40+L40*M40+N40*O40+P40*Q40+R40*S40+T40*U40</f>
         <v>0.57</v>
       </c>
-      <c r="W40" s="15"/>
-      <c r="Y40" s="6"/>
+      <c r="W40" s="16"/>
+      <c r="X40" s="16"/>
+      <c r="Y40" s="16"/>
+      <c r="AA40" s="6"/>
     </row>
-    <row r="41" s="1" customFormat="1" customHeight="1" spans="1:25">
-      <c r="A41" s="15" t="s">
-        <v>45</v>
-      </c>
-      <c r="B41" s="15"/>
-      <c r="C41" s="15" t="s">
-        <v>46</v>
-      </c>
-      <c r="D41" s="31">
-        <f>SUM(D3:D40)</f>
+    <row r="41" s="1" customFormat="1" customHeight="1" spans="1:27">
+      <c r="A41" s="16" t="s">
+        <v>47</v>
+      </c>
+      <c r="B41" s="16"/>
+      <c r="C41" s="16" t="s">
+        <v>48</v>
+      </c>
+      <c r="D41" s="32">
+        <f t="shared" ref="D41:I41" si="5">SUM(D3:D40)</f>
         <v>13</v>
       </c>
-      <c r="E41" s="31">
-        <f>SUM(E3:E40)</f>
+      <c r="E41" s="32">
+        <f t="shared" si="5"/>
         <v>0.84</v>
       </c>
-      <c r="F41" s="31">
-        <f>SUM(F3:F40)</f>
+      <c r="F41" s="32">
+        <f t="shared" si="5"/>
         <v>27</v>
       </c>
-      <c r="G41" s="31">
-        <f>SUM(G3:G40)</f>
+      <c r="G41" s="32">
+        <f t="shared" si="5"/>
         <v>0.95</v>
       </c>
-      <c r="H41" s="31">
-        <f>SUM(H3:H40)</f>
+      <c r="H41" s="32">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="I41" s="31">
-        <f>SUM(I3:I40)</f>
+      <c r="I41" s="32">
+        <f t="shared" si="5"/>
         <v>0</v>
       </c>
-      <c r="J41" s="31">
-        <f t="shared" ref="J41:T41" si="5">SUM(J3:J40)</f>
+      <c r="J41" s="32">
+        <f t="shared" ref="J41:X41" si="6">SUM(J3:J40)</f>
         <v>14</v>
       </c>
-      <c r="K41" s="31">
-        <f t="shared" si="5"/>
+      <c r="K41" s="32">
+        <f t="shared" si="6"/>
         <v>0.72</v>
       </c>
-      <c r="L41" s="31">
-        <f t="shared" si="5"/>
+      <c r="L41" s="32">
+        <f t="shared" si="6"/>
         <v>17</v>
       </c>
-      <c r="M41" s="31">
-        <f t="shared" si="5"/>
+      <c r="M41" s="32">
+        <f t="shared" si="6"/>
         <v>0.55</v>
       </c>
-      <c r="N41" s="31">
-        <f t="shared" si="5"/>
+      <c r="N41" s="32">
+        <f t="shared" si="6"/>
         <v>2</v>
       </c>
-      <c r="O41" s="31">
-        <f t="shared" si="5"/>
+      <c r="O41" s="32">
+        <f t="shared" si="6"/>
         <v>0.12</v>
       </c>
-      <c r="P41" s="31">
-        <f t="shared" si="5"/>
+      <c r="P41" s="32">
+        <f t="shared" si="6"/>
         <v>7</v>
       </c>
-      <c r="Q41" s="31">
-        <f t="shared" si="5"/>
+      <c r="Q41" s="32">
+        <f t="shared" si="6"/>
         <v>0.6</v>
       </c>
-      <c r="R41" s="31">
-        <f t="shared" si="5"/>
+      <c r="R41" s="32">
+        <f t="shared" si="6"/>
         <v>12</v>
       </c>
-      <c r="S41" s="31">
-        <f t="shared" si="5"/>
+      <c r="S41" s="32">
+        <f t="shared" si="6"/>
         <v>0.4</v>
       </c>
-      <c r="T41" s="31">
-        <f>SUM(T3:T40)</f>
+      <c r="T41" s="32">
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="U41" s="31">
-        <f>SUM(U3:U40)</f>
+      <c r="U41" s="32">
+        <f t="shared" si="6"/>
         <v>0</v>
       </c>
-      <c r="V41" s="31">
-        <f>SUM(V3:V40)</f>
+      <c r="V41" s="32">
+        <f t="shared" si="6"/>
         <v>8.34</v>
       </c>
-      <c r="W41" s="15"/>
-      <c r="Y41" s="6"/>
+      <c r="W41" s="32">
+        <f t="shared" si="6"/>
+        <v>0.02</v>
+      </c>
+      <c r="X41" s="32">
+        <f t="shared" si="6"/>
+        <v>0.28</v>
+      </c>
+      <c r="Y41" s="16"/>
+      <c r="AA41" s="6"/>
     </row>
-    <row r="42" customHeight="1" spans="1:25">
-      <c r="A42" s="32"/>
-      <c r="B42" s="32"/>
+    <row r="42" customHeight="1" spans="1:27">
+      <c r="A42" s="33"/>
+      <c r="B42" s="33"/>
     </row>
-    <row r="43" customHeight="1" spans="1:25">
+    <row r="43" customHeight="1" spans="1:27">
       <c r="A43" s="5" t="s">
-        <v>47</v>
+        <v>49</v>
       </c>
     </row>
   </sheetData>
   <mergeCells count="1">
-    <mergeCell ref="A1:W1"/>
+    <mergeCell ref="A1:Y1"/>
   </mergeCells>
   <pageMargins left="0.984027777777778" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
   <pageSetup paperSize="9" scale="37" orientation="portrait"/>

</xml_diff>